<commit_message>
Sync dashboard updates from local project
</commit_message>
<xml_diff>
--- a/backend/data/Daywise Data.xlsx
+++ b/backend/data/Daywise Data.xlsx
@@ -189,7 +189,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:W656"/>
+  <dimension ref="A1:W713"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" bestFit="1" width="13" customWidth="1"/>
@@ -1358,13 +1358,13 @@
         <v>45586</v>
       </c>
       <c r="B17" s="3">
-        <v>68880</v>
+        <v>67200</v>
       </c>
       <c r="C17" s="3">
         <v>1680</v>
       </c>
       <c r="D17" s="3">
-        <v>16800</v>
+        <v>18480</v>
       </c>
       <c r="E17" s="3">
         <v>0</v>
@@ -1373,10 +1373,10 @@
         <v>87360</v>
       </c>
       <c r="G17" s="3">
+        <v>0</v>
+      </c>
+      <c r="H17" s="3">
         <v>1440</v>
-      </c>
-      <c r="H17" s="3">
-        <v>0</v>
       </c>
       <c r="I17" s="3">
         <v>0</v>
@@ -1403,22 +1403,22 @@
         <v>2776</v>
       </c>
       <c r="Q17" s="4">
-        <v>75.216</v>
+        <v>73.382</v>
       </c>
       <c r="R17" s="4">
         <v>1.835</v>
       </c>
       <c r="S17" s="4">
-        <v>18.345</v>
+        <v>20.180</v>
       </c>
       <c r="T17" s="3">
         <v>0</v>
       </c>
-      <c r="U17" s="4">
+      <c r="U17" s="3">
+        <v>0</v>
+      </c>
+      <c r="V17" s="4">
         <v>1.572</v>
-      </c>
-      <c r="V17" s="3">
-        <v>0</v>
       </c>
       <c r="W17" s="4">
         <v>3.031</v>
@@ -1855,13 +1855,13 @@
         <v>45593</v>
       </c>
       <c r="B24" s="3">
-        <v>14160</v>
+        <v>12480</v>
       </c>
       <c r="C24" s="3">
         <v>10560</v>
       </c>
       <c r="D24" s="3">
-        <v>99720</v>
+        <v>101400</v>
       </c>
       <c r="E24" s="3">
         <v>3360</v>
@@ -1900,13 +1900,13 @@
         <v>1978</v>
       </c>
       <c r="Q24" s="4">
-        <v>10.522</v>
+        <v>9.273</v>
       </c>
       <c r="R24" s="4">
         <v>7.847</v>
       </c>
       <c r="S24" s="4">
-        <v>74.098</v>
+        <v>75.347</v>
       </c>
       <c r="T24" s="4">
         <v>2.497</v>
@@ -2352,13 +2352,13 @@
         <v>45600</v>
       </c>
       <c r="B31" s="3">
-        <v>100920</v>
+        <v>102600</v>
       </c>
       <c r="C31" s="3">
         <v>1560</v>
       </c>
       <c r="D31" s="3">
-        <v>27960</v>
+        <v>26280</v>
       </c>
       <c r="E31" s="3">
         <v>1560</v>
@@ -2397,13 +2397,13 @@
         <v>2556</v>
       </c>
       <c r="Q31" s="4">
-        <v>75.002</v>
+        <v>76.251</v>
       </c>
       <c r="R31" s="4">
         <v>1.159</v>
       </c>
       <c r="S31" s="4">
-        <v>20.779</v>
+        <v>19.531</v>
       </c>
       <c r="T31" s="4">
         <v>1.159</v>
@@ -2494,13 +2494,13 @@
         <v>45602</v>
       </c>
       <c r="B33" s="3">
-        <v>136920</v>
+        <v>135480</v>
       </c>
       <c r="C33" s="3">
         <v>1680</v>
       </c>
       <c r="D33" s="3">
-        <v>15240</v>
+        <v>16680</v>
       </c>
       <c r="E33" s="3">
         <v>0</v>
@@ -2539,13 +2539,13 @@
         <v>1888</v>
       </c>
       <c r="Q33" s="4">
-        <v>87.923</v>
+        <v>86.998</v>
       </c>
       <c r="R33" s="4">
         <v>1.079</v>
       </c>
       <c r="S33" s="4">
-        <v>9.786</v>
+        <v>10.711</v>
       </c>
       <c r="T33" s="3">
         <v>0</v>
@@ -46727,19 +46727,19 @@
         <v>46227</v>
       </c>
       <c r="B656" s="3">
-        <v>446740</v>
+        <v>716380</v>
       </c>
       <c r="C656" s="3">
-        <v>0</v>
+        <v>7280</v>
       </c>
       <c r="D656" s="3">
-        <v>19600</v>
+        <v>54320</v>
       </c>
       <c r="E656" s="3">
-        <v>1960</v>
+        <v>3360</v>
       </c>
       <c r="F656" s="3">
-        <v>468300</v>
+        <v>781340</v>
       </c>
       <c r="G656" s="3">
         <v>1960</v>
@@ -46754,43 +46754,4090 @@
         <v>7840</v>
       </c>
       <c r="K656" s="3">
-        <v>1958</v>
+        <v>2896</v>
       </c>
       <c r="L656" s="3">
-        <v>1814</v>
+        <v>2964</v>
       </c>
       <c r="M656" s="3">
-        <v>285</v>
+        <v>387</v>
       </c>
       <c r="N656" s="3">
-        <v>365</v>
+        <v>625</v>
       </c>
       <c r="O656" s="3">
-        <v>1727</v>
+        <v>2503</v>
       </c>
       <c r="P656" s="3">
-        <v>6149</v>
+        <v>9375</v>
       </c>
       <c r="Q656" s="4">
-        <v>92.629</v>
-      </c>
-      <c r="R656" s="3">
-        <v>0</v>
+        <v>89.710</v>
+      </c>
+      <c r="R656" s="4">
+        <v>0.912</v>
       </c>
       <c r="S656" s="4">
-        <v>4.064</v>
+        <v>6.802</v>
       </c>
       <c r="T656" s="4">
-        <v>0.406</v>
+        <v>0.421</v>
       </c>
       <c r="U656" s="4">
-        <v>0.813</v>
+        <v>0.491</v>
       </c>
       <c r="V656" s="4">
-        <v>0.813</v>
+        <v>0.491</v>
       </c>
       <c r="W656" s="4">
-        <v>1.275</v>
+        <v>1.174</v>
+      </c>
+    </row>
+    <row r="657" spans="1:23">
+      <c r="A657" s="2">
+        <v>46228</v>
+      </c>
+      <c r="B657" s="3">
+        <v>707560</v>
+      </c>
+      <c r="C657" s="3">
+        <v>2940</v>
+      </c>
+      <c r="D657" s="3">
+        <v>58340</v>
+      </c>
+      <c r="E657" s="3">
+        <v>3640</v>
+      </c>
+      <c r="F657" s="3">
+        <v>772480</v>
+      </c>
+      <c r="G657" s="3">
+        <v>0</v>
+      </c>
+      <c r="H657" s="3">
+        <v>7840</v>
+      </c>
+      <c r="I657" s="3">
+        <v>3920</v>
+      </c>
+      <c r="J657" s="3">
+        <v>11760</v>
+      </c>
+      <c r="K657" s="3">
+        <v>2678</v>
+      </c>
+      <c r="L657" s="3">
+        <v>3391</v>
+      </c>
+      <c r="M657" s="3">
+        <v>289</v>
+      </c>
+      <c r="N657" s="3">
+        <v>581</v>
+      </c>
+      <c r="O657" s="3">
+        <v>2901</v>
+      </c>
+      <c r="P657" s="3">
+        <v>9840</v>
+      </c>
+      <c r="Q657" s="4">
+        <v>89.104</v>
+      </c>
+      <c r="R657" s="4">
+        <v>0.370</v>
+      </c>
+      <c r="S657" s="4">
+        <v>7.347</v>
+      </c>
+      <c r="T657" s="4">
+        <v>0.458</v>
+      </c>
+      <c r="U657" s="3">
+        <v>0</v>
+      </c>
+      <c r="V657" s="4">
+        <v>0.987</v>
+      </c>
+      <c r="W657" s="4">
+        <v>1.239</v>
+      </c>
+    </row>
+    <row r="658" spans="1:23">
+      <c r="A658" s="2">
+        <v>46229</v>
+      </c>
+      <c r="B658" s="3">
+        <v>692580</v>
+      </c>
+      <c r="C658" s="3">
+        <v>7280</v>
+      </c>
+      <c r="D658" s="3">
+        <v>55020</v>
+      </c>
+      <c r="E658" s="3">
+        <v>3920</v>
+      </c>
+      <c r="F658" s="3">
+        <v>758800</v>
+      </c>
+      <c r="G658" s="3">
+        <v>1960</v>
+      </c>
+      <c r="H658" s="3">
+        <v>3920</v>
+      </c>
+      <c r="I658" s="3">
+        <v>1960</v>
+      </c>
+      <c r="J658" s="3">
+        <v>7840</v>
+      </c>
+      <c r="K658" s="3">
+        <v>2499</v>
+      </c>
+      <c r="L658" s="3">
+        <v>3088</v>
+      </c>
+      <c r="M658" s="3">
+        <v>338</v>
+      </c>
+      <c r="N658" s="3">
+        <v>560</v>
+      </c>
+      <c r="O658" s="3">
+        <v>2810</v>
+      </c>
+      <c r="P658" s="3">
+        <v>9295</v>
+      </c>
+      <c r="Q658" s="4">
+        <v>89.257</v>
+      </c>
+      <c r="R658" s="4">
+        <v>0.938</v>
+      </c>
+      <c r="S658" s="4">
+        <v>7.091</v>
+      </c>
+      <c r="T658" s="4">
+        <v>0.505</v>
+      </c>
+      <c r="U658" s="4">
+        <v>0.505</v>
+      </c>
+      <c r="V658" s="4">
+        <v>0.505</v>
+      </c>
+      <c r="W658" s="4">
+        <v>1.198</v>
+      </c>
+    </row>
+    <row r="659" spans="1:23">
+      <c r="A659" s="2">
+        <v>46230</v>
+      </c>
+      <c r="B659" s="3">
+        <v>698880</v>
+      </c>
+      <c r="C659" s="3">
+        <v>5320</v>
+      </c>
+      <c r="D659" s="3">
+        <v>59080</v>
+      </c>
+      <c r="E659" s="3">
+        <v>3920</v>
+      </c>
+      <c r="F659" s="3">
+        <v>767200</v>
+      </c>
+      <c r="G659" s="3">
+        <v>3920</v>
+      </c>
+      <c r="H659" s="3">
+        <v>3920</v>
+      </c>
+      <c r="I659" s="3">
+        <v>0</v>
+      </c>
+      <c r="J659" s="3">
+        <v>7840</v>
+      </c>
+      <c r="K659" s="3">
+        <v>3121</v>
+      </c>
+      <c r="L659" s="3">
+        <v>3047</v>
+      </c>
+      <c r="M659" s="3">
+        <v>243</v>
+      </c>
+      <c r="N659" s="3">
+        <v>636</v>
+      </c>
+      <c r="O659" s="3">
+        <v>2479</v>
+      </c>
+      <c r="P659" s="3">
+        <v>9526</v>
+      </c>
+      <c r="Q659" s="4">
+        <v>89.079</v>
+      </c>
+      <c r="R659" s="4">
+        <v>0.678</v>
+      </c>
+      <c r="S659" s="4">
+        <v>7.530</v>
+      </c>
+      <c r="T659" s="4">
+        <v>0.500</v>
+      </c>
+      <c r="U659" s="4">
+        <v>0.500</v>
+      </c>
+      <c r="V659" s="4">
+        <v>0.500</v>
+      </c>
+      <c r="W659" s="4">
+        <v>1.214</v>
+      </c>
+    </row>
+    <row r="660" spans="1:23">
+      <c r="A660" s="2">
+        <v>46231</v>
+      </c>
+      <c r="B660" s="3">
+        <v>680680</v>
+      </c>
+      <c r="C660" s="3">
+        <v>5320</v>
+      </c>
+      <c r="D660" s="3">
+        <v>68180</v>
+      </c>
+      <c r="E660" s="3">
+        <v>3500</v>
+      </c>
+      <c r="F660" s="3">
+        <v>757680</v>
+      </c>
+      <c r="G660" s="3">
+        <v>1960</v>
+      </c>
+      <c r="H660" s="3">
+        <v>3920</v>
+      </c>
+      <c r="I660" s="3">
+        <v>1960</v>
+      </c>
+      <c r="J660" s="3">
+        <v>7840</v>
+      </c>
+      <c r="K660" s="3">
+        <v>2939</v>
+      </c>
+      <c r="L660" s="3">
+        <v>3368</v>
+      </c>
+      <c r="M660" s="3">
+        <v>281</v>
+      </c>
+      <c r="N660" s="3">
+        <v>525</v>
+      </c>
+      <c r="O660" s="3">
+        <v>2417</v>
+      </c>
+      <c r="P660" s="3">
+        <v>9530</v>
+      </c>
+      <c r="Q660" s="4">
+        <v>87.824</v>
+      </c>
+      <c r="R660" s="4">
+        <v>0.686</v>
+      </c>
+      <c r="S660" s="4">
+        <v>8.797</v>
+      </c>
+      <c r="T660" s="4">
+        <v>0.452</v>
+      </c>
+      <c r="U660" s="4">
+        <v>0.506</v>
+      </c>
+      <c r="V660" s="4">
+        <v>0.506</v>
+      </c>
+      <c r="W660" s="4">
+        <v>1.230</v>
+      </c>
+    </row>
+    <row r="661" spans="1:23">
+      <c r="A661" s="2">
+        <v>46232</v>
+      </c>
+      <c r="B661" s="3">
+        <v>685300</v>
+      </c>
+      <c r="C661" s="3">
+        <v>4900</v>
+      </c>
+      <c r="D661" s="3">
+        <v>82460</v>
+      </c>
+      <c r="E661" s="3">
+        <v>5600</v>
+      </c>
+      <c r="F661" s="3">
+        <v>778260</v>
+      </c>
+      <c r="G661" s="3">
+        <v>1960</v>
+      </c>
+      <c r="H661" s="3">
+        <v>3920</v>
+      </c>
+      <c r="I661" s="3">
+        <v>1960</v>
+      </c>
+      <c r="J661" s="3">
+        <v>7840</v>
+      </c>
+      <c r="K661" s="3">
+        <v>3605</v>
+      </c>
+      <c r="L661" s="3">
+        <v>2993</v>
+      </c>
+      <c r="M661" s="3">
+        <v>242</v>
+      </c>
+      <c r="N661" s="3">
+        <v>668</v>
+      </c>
+      <c r="O661" s="3">
+        <v>2814</v>
+      </c>
+      <c r="P661" s="3">
+        <v>10322</v>
+      </c>
+      <c r="Q661" s="4">
+        <v>86.047</v>
+      </c>
+      <c r="R661" s="4">
+        <v>0.615</v>
+      </c>
+      <c r="S661" s="4">
+        <v>10.354</v>
+      </c>
+      <c r="T661" s="4">
+        <v>0.703</v>
+      </c>
+      <c r="U661" s="4">
+        <v>0.492</v>
+      </c>
+      <c r="V661" s="4">
+        <v>0.492</v>
+      </c>
+      <c r="W661" s="4">
+        <v>1.296</v>
+      </c>
+    </row>
+    <row r="662" spans="1:23">
+      <c r="A662" s="2">
+        <v>46233</v>
+      </c>
+      <c r="B662" s="3">
+        <v>692300</v>
+      </c>
+      <c r="C662" s="3">
+        <v>9660</v>
+      </c>
+      <c r="D662" s="3">
+        <v>85260</v>
+      </c>
+      <c r="E662" s="3">
+        <v>3780</v>
+      </c>
+      <c r="F662" s="3">
+        <v>791000</v>
+      </c>
+      <c r="G662" s="3">
+        <v>1960</v>
+      </c>
+      <c r="H662" s="3">
+        <v>3920</v>
+      </c>
+      <c r="I662" s="3">
+        <v>0</v>
+      </c>
+      <c r="J662" s="3">
+        <v>5880</v>
+      </c>
+      <c r="K662" s="3">
+        <v>2849</v>
+      </c>
+      <c r="L662" s="3">
+        <v>3208</v>
+      </c>
+      <c r="M662" s="3">
+        <v>275</v>
+      </c>
+      <c r="N662" s="3">
+        <v>653</v>
+      </c>
+      <c r="O662" s="3">
+        <v>2455</v>
+      </c>
+      <c r="P662" s="3">
+        <v>9440</v>
+      </c>
+      <c r="Q662" s="4">
+        <v>85.859</v>
+      </c>
+      <c r="R662" s="4">
+        <v>1.198</v>
+      </c>
+      <c r="S662" s="4">
+        <v>10.574</v>
+      </c>
+      <c r="T662" s="4">
+        <v>0.469</v>
+      </c>
+      <c r="U662" s="4">
+        <v>0.243</v>
+      </c>
+      <c r="V662" s="4">
+        <v>0.486</v>
+      </c>
+      <c r="W662" s="4">
+        <v>1.171</v>
+      </c>
+    </row>
+    <row r="663" spans="1:23">
+      <c r="A663" s="2">
+        <v>46234</v>
+      </c>
+      <c r="B663" s="3">
+        <v>681940</v>
+      </c>
+      <c r="C663" s="3">
+        <v>9240</v>
+      </c>
+      <c r="D663" s="3">
+        <v>83720</v>
+      </c>
+      <c r="E663" s="3">
+        <v>4900</v>
+      </c>
+      <c r="F663" s="3">
+        <v>779800</v>
+      </c>
+      <c r="G663" s="3">
+        <v>3920</v>
+      </c>
+      <c r="H663" s="3">
+        <v>3920</v>
+      </c>
+      <c r="I663" s="3">
+        <v>0</v>
+      </c>
+      <c r="J663" s="3">
+        <v>7840</v>
+      </c>
+      <c r="K663" s="3">
+        <v>2828</v>
+      </c>
+      <c r="L663" s="3">
+        <v>3522</v>
+      </c>
+      <c r="M663" s="3">
+        <v>402</v>
+      </c>
+      <c r="N663" s="3">
+        <v>644</v>
+      </c>
+      <c r="O663" s="3">
+        <v>2250</v>
+      </c>
+      <c r="P663" s="3">
+        <v>9646</v>
+      </c>
+      <c r="Q663" s="4">
+        <v>85.533</v>
+      </c>
+      <c r="R663" s="4">
+        <v>1.159</v>
+      </c>
+      <c r="S663" s="4">
+        <v>10.501</v>
+      </c>
+      <c r="T663" s="4">
+        <v>0.615</v>
+      </c>
+      <c r="U663" s="4">
+        <v>0.492</v>
+      </c>
+      <c r="V663" s="4">
+        <v>0.492</v>
+      </c>
+      <c r="W663" s="4">
+        <v>1.210</v>
+      </c>
+    </row>
+    <row r="664" spans="1:23">
+      <c r="A664" s="2">
+        <v>46235</v>
+      </c>
+      <c r="B664" s="3">
+        <v>397420</v>
+      </c>
+      <c r="C664" s="3">
+        <v>0</v>
+      </c>
+      <c r="D664" s="3">
+        <v>94920</v>
+      </c>
+      <c r="E664" s="3">
+        <v>3640</v>
+      </c>
+      <c r="F664" s="3">
+        <v>495980</v>
+      </c>
+      <c r="G664" s="3">
+        <v>5880</v>
+      </c>
+      <c r="H664" s="3">
+        <v>1960</v>
+      </c>
+      <c r="I664" s="3">
+        <v>0</v>
+      </c>
+      <c r="J664" s="3">
+        <v>7840</v>
+      </c>
+      <c r="K664" s="3">
+        <v>6934</v>
+      </c>
+      <c r="L664" s="3">
+        <v>4495</v>
+      </c>
+      <c r="M664" s="3">
+        <v>559</v>
+      </c>
+      <c r="N664" s="3">
+        <v>715</v>
+      </c>
+      <c r="O664" s="3">
+        <v>3055</v>
+      </c>
+      <c r="P664" s="3">
+        <v>15758</v>
+      </c>
+      <c r="Q664" s="4">
+        <v>76.489</v>
+      </c>
+      <c r="R664" s="3">
+        <v>0</v>
+      </c>
+      <c r="S664" s="4">
+        <v>18.269</v>
+      </c>
+      <c r="T664" s="4">
+        <v>0.701</v>
+      </c>
+      <c r="U664" s="4">
+        <v>1.132</v>
+      </c>
+      <c r="V664" s="4">
+        <v>0.377</v>
+      </c>
+      <c r="W664" s="4">
+        <v>3.033</v>
+      </c>
+    </row>
+    <row r="665" spans="1:23">
+      <c r="A665" s="2">
+        <v>46236</v>
+      </c>
+      <c r="B665" s="3">
+        <v>339500</v>
+      </c>
+      <c r="C665" s="3">
+        <v>5740</v>
+      </c>
+      <c r="D665" s="3">
+        <v>236180</v>
+      </c>
+      <c r="E665" s="3">
+        <v>12880</v>
+      </c>
+      <c r="F665" s="3">
+        <v>594300</v>
+      </c>
+      <c r="G665" s="3">
+        <v>13720</v>
+      </c>
+      <c r="H665" s="3">
+        <v>1960</v>
+      </c>
+      <c r="I665" s="3">
+        <v>1960</v>
+      </c>
+      <c r="J665" s="3">
+        <v>17640</v>
+      </c>
+      <c r="K665" s="3">
+        <v>2285</v>
+      </c>
+      <c r="L665" s="3">
+        <v>3184</v>
+      </c>
+      <c r="M665" s="3">
+        <v>322</v>
+      </c>
+      <c r="N665" s="3">
+        <v>660</v>
+      </c>
+      <c r="O665" s="3">
+        <v>2044</v>
+      </c>
+      <c r="P665" s="3">
+        <v>8495</v>
+      </c>
+      <c r="Q665" s="4">
+        <v>54.720</v>
+      </c>
+      <c r="R665" s="4">
+        <v>0.925</v>
+      </c>
+      <c r="S665" s="4">
+        <v>38.067</v>
+      </c>
+      <c r="T665" s="4">
+        <v>2.076</v>
+      </c>
+      <c r="U665" s="4">
+        <v>2.527</v>
+      </c>
+      <c r="V665" s="4">
+        <v>0.316</v>
+      </c>
+      <c r="W665" s="4">
+        <v>1.369</v>
+      </c>
+    </row>
+    <row r="666" spans="1:23">
+      <c r="A666" s="2">
+        <v>46237</v>
+      </c>
+      <c r="B666" s="3">
+        <v>635320</v>
+      </c>
+      <c r="C666" s="3">
+        <v>5460</v>
+      </c>
+      <c r="D666" s="3">
+        <v>111780</v>
+      </c>
+      <c r="E666" s="3">
+        <v>0</v>
+      </c>
+      <c r="F666" s="3">
+        <v>752560</v>
+      </c>
+      <c r="G666" s="3">
+        <v>3920</v>
+      </c>
+      <c r="H666" s="3">
+        <v>1960</v>
+      </c>
+      <c r="I666" s="3">
+        <v>0</v>
+      </c>
+      <c r="J666" s="3">
+        <v>5880</v>
+      </c>
+      <c r="K666" s="3">
+        <v>2791</v>
+      </c>
+      <c r="L666" s="3">
+        <v>3095</v>
+      </c>
+      <c r="M666" s="3">
+        <v>320</v>
+      </c>
+      <c r="N666" s="3">
+        <v>716</v>
+      </c>
+      <c r="O666" s="3">
+        <v>2279</v>
+      </c>
+      <c r="P666" s="3">
+        <v>9201</v>
+      </c>
+      <c r="Q666" s="4">
+        <v>82.763</v>
+      </c>
+      <c r="R666" s="4">
+        <v>0.711</v>
+      </c>
+      <c r="S666" s="4">
+        <v>14.561</v>
+      </c>
+      <c r="T666" s="3">
+        <v>0</v>
+      </c>
+      <c r="U666" s="4">
+        <v>0.511</v>
+      </c>
+      <c r="V666" s="4">
+        <v>0.255</v>
+      </c>
+      <c r="W666" s="4">
+        <v>1.199</v>
+      </c>
+    </row>
+    <row r="667" spans="1:23">
+      <c r="A667" s="2">
+        <v>46238</v>
+      </c>
+      <c r="B667" s="3">
+        <v>656880</v>
+      </c>
+      <c r="C667" s="3">
+        <v>9100</v>
+      </c>
+      <c r="D667" s="3">
+        <v>102620</v>
+      </c>
+      <c r="E667" s="3">
+        <v>3920</v>
+      </c>
+      <c r="F667" s="3">
+        <v>772520</v>
+      </c>
+      <c r="G667" s="3">
+        <v>3920</v>
+      </c>
+      <c r="H667" s="3">
+        <v>1960</v>
+      </c>
+      <c r="I667" s="3">
+        <v>1960</v>
+      </c>
+      <c r="J667" s="3">
+        <v>7840</v>
+      </c>
+      <c r="K667" s="3">
+        <v>2530</v>
+      </c>
+      <c r="L667" s="3">
+        <v>3644</v>
+      </c>
+      <c r="M667" s="3">
+        <v>252</v>
+      </c>
+      <c r="N667" s="3">
+        <v>591</v>
+      </c>
+      <c r="O667" s="3">
+        <v>2388</v>
+      </c>
+      <c r="P667" s="3">
+        <v>9405</v>
+      </c>
+      <c r="Q667" s="4">
+        <v>83.174</v>
+      </c>
+      <c r="R667" s="4">
+        <v>1.152</v>
+      </c>
+      <c r="S667" s="4">
+        <v>12.994</v>
+      </c>
+      <c r="T667" s="4">
+        <v>0.496</v>
+      </c>
+      <c r="U667" s="4">
+        <v>0.745</v>
+      </c>
+      <c r="V667" s="4">
+        <v>0.248</v>
+      </c>
+      <c r="W667" s="4">
+        <v>1.191</v>
+      </c>
+    </row>
+    <row r="668" spans="1:23">
+      <c r="A668" s="2">
+        <v>46239</v>
+      </c>
+      <c r="B668" s="3">
+        <v>488040</v>
+      </c>
+      <c r="C668" s="3">
+        <v>6860</v>
+      </c>
+      <c r="D668" s="3">
+        <v>233900</v>
+      </c>
+      <c r="E668" s="3">
+        <v>11760</v>
+      </c>
+      <c r="F668" s="3">
+        <v>740560</v>
+      </c>
+      <c r="G668" s="3">
+        <v>5880</v>
+      </c>
+      <c r="H668" s="3">
+        <v>3920</v>
+      </c>
+      <c r="I668" s="3">
+        <v>0</v>
+      </c>
+      <c r="J668" s="3">
+        <v>9800</v>
+      </c>
+      <c r="K668" s="3">
+        <v>2515</v>
+      </c>
+      <c r="L668" s="3">
+        <v>3217</v>
+      </c>
+      <c r="M668" s="3">
+        <v>918</v>
+      </c>
+      <c r="N668" s="3">
+        <v>639</v>
+      </c>
+      <c r="O668" s="3">
+        <v>2211</v>
+      </c>
+      <c r="P668" s="3">
+        <v>9500</v>
+      </c>
+      <c r="Q668" s="4">
+        <v>64.228</v>
+      </c>
+      <c r="R668" s="4">
+        <v>0.903</v>
+      </c>
+      <c r="S668" s="4">
+        <v>30.782</v>
+      </c>
+      <c r="T668" s="4">
+        <v>1.548</v>
+      </c>
+      <c r="U668" s="4">
+        <v>0.774</v>
+      </c>
+      <c r="V668" s="4">
+        <v>0.516</v>
+      </c>
+      <c r="W668" s="4">
+        <v>1.250</v>
+      </c>
+    </row>
+    <row r="669" spans="1:23">
+      <c r="A669" s="2">
+        <v>46240</v>
+      </c>
+      <c r="B669" s="3">
+        <v>536900</v>
+      </c>
+      <c r="C669" s="3">
+        <v>7840</v>
+      </c>
+      <c r="D669" s="3">
+        <v>169540</v>
+      </c>
+      <c r="E669" s="3">
+        <v>3780</v>
+      </c>
+      <c r="F669" s="3">
+        <v>718060</v>
+      </c>
+      <c r="G669" s="3">
+        <v>3640</v>
+      </c>
+      <c r="H669" s="3">
+        <v>1960</v>
+      </c>
+      <c r="I669" s="3">
+        <v>1960</v>
+      </c>
+      <c r="J669" s="3">
+        <v>7560</v>
+      </c>
+      <c r="K669" s="3">
+        <v>2713</v>
+      </c>
+      <c r="L669" s="3">
+        <v>4174</v>
+      </c>
+      <c r="M669" s="3">
+        <v>296</v>
+      </c>
+      <c r="N669" s="3">
+        <v>672</v>
+      </c>
+      <c r="O669" s="3">
+        <v>2322</v>
+      </c>
+      <c r="P669" s="3">
+        <v>10177</v>
+      </c>
+      <c r="Q669" s="4">
+        <v>72.968</v>
+      </c>
+      <c r="R669" s="4">
+        <v>1.066</v>
+      </c>
+      <c r="S669" s="4">
+        <v>23.042</v>
+      </c>
+      <c r="T669" s="4">
+        <v>0.514</v>
+      </c>
+      <c r="U669" s="4">
+        <v>0.761</v>
+      </c>
+      <c r="V669" s="4">
+        <v>0.266</v>
+      </c>
+      <c r="W669" s="4">
+        <v>1.383</v>
+      </c>
+    </row>
+    <row r="670" spans="1:23">
+      <c r="A670" s="2">
+        <v>46241</v>
+      </c>
+      <c r="B670" s="3">
+        <v>649460</v>
+      </c>
+      <c r="C670" s="3">
+        <v>9240</v>
+      </c>
+      <c r="D670" s="3">
+        <v>59700</v>
+      </c>
+      <c r="E670" s="3">
+        <v>3920</v>
+      </c>
+      <c r="F670" s="3">
+        <v>722320</v>
+      </c>
+      <c r="G670" s="3">
+        <v>1960</v>
+      </c>
+      <c r="H670" s="3">
+        <v>1960</v>
+      </c>
+      <c r="I670" s="3">
+        <v>0</v>
+      </c>
+      <c r="J670" s="3">
+        <v>3920</v>
+      </c>
+      <c r="K670" s="3">
+        <v>2708</v>
+      </c>
+      <c r="L670" s="3">
+        <v>3273</v>
+      </c>
+      <c r="M670" s="3">
+        <v>464</v>
+      </c>
+      <c r="N670" s="3">
+        <v>895</v>
+      </c>
+      <c r="O670" s="3">
+        <v>2252</v>
+      </c>
+      <c r="P670" s="3">
+        <v>9592</v>
+      </c>
+      <c r="Q670" s="4">
+        <v>88.262</v>
+      </c>
+      <c r="R670" s="4">
+        <v>1.256</v>
+      </c>
+      <c r="S670" s="4">
+        <v>8.113</v>
+      </c>
+      <c r="T670" s="4">
+        <v>0.533</v>
+      </c>
+      <c r="U670" s="4">
+        <v>0.266</v>
+      </c>
+      <c r="V670" s="4">
+        <v>0.266</v>
+      </c>
+      <c r="W670" s="4">
+        <v>1.304</v>
+      </c>
+    </row>
+    <row r="671" spans="1:23">
+      <c r="A671" s="2">
+        <v>46242</v>
+      </c>
+      <c r="B671" s="3">
+        <v>637560</v>
+      </c>
+      <c r="C671" s="3">
+        <v>8260</v>
+      </c>
+      <c r="D671" s="3">
+        <v>63980</v>
+      </c>
+      <c r="E671" s="3">
+        <v>5460</v>
+      </c>
+      <c r="F671" s="3">
+        <v>715260</v>
+      </c>
+      <c r="G671" s="3">
+        <v>3500</v>
+      </c>
+      <c r="H671" s="3">
+        <v>0</v>
+      </c>
+      <c r="I671" s="3">
+        <v>1540</v>
+      </c>
+      <c r="J671" s="3">
+        <v>5040</v>
+      </c>
+      <c r="K671" s="3">
+        <v>3451</v>
+      </c>
+      <c r="L671" s="3">
+        <v>3434</v>
+      </c>
+      <c r="M671" s="3">
+        <v>374</v>
+      </c>
+      <c r="N671" s="3">
+        <v>623</v>
+      </c>
+      <c r="O671" s="3">
+        <v>2604</v>
+      </c>
+      <c r="P671" s="3">
+        <v>10486</v>
+      </c>
+      <c r="Q671" s="4">
+        <v>87.243</v>
+      </c>
+      <c r="R671" s="4">
+        <v>1.130</v>
+      </c>
+      <c r="S671" s="4">
+        <v>8.755</v>
+      </c>
+      <c r="T671" s="4">
+        <v>0.747</v>
+      </c>
+      <c r="U671" s="4">
+        <v>0.690</v>
+      </c>
+      <c r="V671" s="3">
+        <v>0</v>
+      </c>
+      <c r="W671" s="4">
+        <v>1.435</v>
+      </c>
+    </row>
+    <row r="672" spans="1:23">
+      <c r="A672" s="2">
+        <v>46243</v>
+      </c>
+      <c r="B672" s="3">
+        <v>704480</v>
+      </c>
+      <c r="C672" s="3">
+        <v>9520</v>
+      </c>
+      <c r="D672" s="3">
+        <v>61180</v>
+      </c>
+      <c r="E672" s="3">
+        <v>3920</v>
+      </c>
+      <c r="F672" s="3">
+        <v>779100</v>
+      </c>
+      <c r="G672" s="3">
+        <v>3920</v>
+      </c>
+      <c r="H672" s="3">
+        <v>0</v>
+      </c>
+      <c r="I672" s="3">
+        <v>0</v>
+      </c>
+      <c r="J672" s="3">
+        <v>3920</v>
+      </c>
+      <c r="K672" s="3">
+        <v>2815</v>
+      </c>
+      <c r="L672" s="3">
+        <v>3116</v>
+      </c>
+      <c r="M672" s="3">
+        <v>336</v>
+      </c>
+      <c r="N672" s="3">
+        <v>563</v>
+      </c>
+      <c r="O672" s="3">
+        <v>2508</v>
+      </c>
+      <c r="P672" s="3">
+        <v>9338</v>
+      </c>
+      <c r="Q672" s="4">
+        <v>88.909</v>
+      </c>
+      <c r="R672" s="4">
+        <v>1.201</v>
+      </c>
+      <c r="S672" s="4">
+        <v>7.721</v>
+      </c>
+      <c r="T672" s="4">
+        <v>0.495</v>
+      </c>
+      <c r="U672" s="4">
+        <v>0.495</v>
+      </c>
+      <c r="V672" s="3">
+        <v>0</v>
+      </c>
+      <c r="W672" s="4">
+        <v>1.179</v>
+      </c>
+    </row>
+    <row r="673" spans="1:23">
+      <c r="A673" s="2">
+        <v>46244</v>
+      </c>
+      <c r="B673" s="3">
+        <v>713720</v>
+      </c>
+      <c r="C673" s="3">
+        <v>8960</v>
+      </c>
+      <c r="D673" s="3">
+        <v>62160</v>
+      </c>
+      <c r="E673" s="3">
+        <v>3640</v>
+      </c>
+      <c r="F673" s="3">
+        <v>788480</v>
+      </c>
+      <c r="G673" s="3">
+        <v>1960</v>
+      </c>
+      <c r="H673" s="3">
+        <v>1960</v>
+      </c>
+      <c r="I673" s="3">
+        <v>0</v>
+      </c>
+      <c r="J673" s="3">
+        <v>3920</v>
+      </c>
+      <c r="K673" s="3">
+        <v>3587</v>
+      </c>
+      <c r="L673" s="3">
+        <v>2812</v>
+      </c>
+      <c r="M673" s="3">
+        <v>374</v>
+      </c>
+      <c r="N673" s="3">
+        <v>514</v>
+      </c>
+      <c r="O673" s="3">
+        <v>2339</v>
+      </c>
+      <c r="P673" s="3">
+        <v>9626</v>
+      </c>
+      <c r="Q673" s="4">
+        <v>88.990</v>
+      </c>
+      <c r="R673" s="4">
+        <v>1.117</v>
+      </c>
+      <c r="S673" s="4">
+        <v>7.750</v>
+      </c>
+      <c r="T673" s="4">
+        <v>0.454</v>
+      </c>
+      <c r="U673" s="4">
+        <v>0.244</v>
+      </c>
+      <c r="V673" s="4">
+        <v>0.244</v>
+      </c>
+      <c r="W673" s="4">
+        <v>1.200</v>
+      </c>
+    </row>
+    <row r="674" spans="1:23">
+      <c r="A674" s="2">
+        <v>46245</v>
+      </c>
+      <c r="B674" s="3">
+        <v>644980</v>
+      </c>
+      <c r="C674" s="3">
+        <v>2940</v>
+      </c>
+      <c r="D674" s="3">
+        <v>79800</v>
+      </c>
+      <c r="E674" s="3">
+        <v>6580</v>
+      </c>
+      <c r="F674" s="3">
+        <v>734300</v>
+      </c>
+      <c r="G674" s="3">
+        <v>1960</v>
+      </c>
+      <c r="H674" s="3">
+        <v>1960</v>
+      </c>
+      <c r="I674" s="3">
+        <v>1960</v>
+      </c>
+      <c r="J674" s="3">
+        <v>5880</v>
+      </c>
+      <c r="K674" s="3">
+        <v>2518</v>
+      </c>
+      <c r="L674" s="3">
+        <v>3743</v>
+      </c>
+      <c r="M674" s="3">
+        <v>389</v>
+      </c>
+      <c r="N674" s="3">
+        <v>746</v>
+      </c>
+      <c r="O674" s="3">
+        <v>2541</v>
+      </c>
+      <c r="P674" s="3">
+        <v>9937</v>
+      </c>
+      <c r="Q674" s="4">
+        <v>85.984</v>
+      </c>
+      <c r="R674" s="4">
+        <v>0.392</v>
+      </c>
+      <c r="S674" s="4">
+        <v>10.638</v>
+      </c>
+      <c r="T674" s="4">
+        <v>0.877</v>
+      </c>
+      <c r="U674" s="4">
+        <v>0.523</v>
+      </c>
+      <c r="V674" s="4">
+        <v>0.261</v>
+      </c>
+      <c r="W674" s="4">
+        <v>1.325</v>
+      </c>
+    </row>
+    <row r="675" spans="1:23">
+      <c r="A675" s="2">
+        <v>46246</v>
+      </c>
+      <c r="B675" s="3">
+        <v>707000</v>
+      </c>
+      <c r="C675" s="3">
+        <v>5180</v>
+      </c>
+      <c r="D675" s="3">
+        <v>50820</v>
+      </c>
+      <c r="E675" s="3">
+        <v>6720</v>
+      </c>
+      <c r="F675" s="3">
+        <v>769720</v>
+      </c>
+      <c r="G675" s="3">
+        <v>3500</v>
+      </c>
+      <c r="H675" s="3">
+        <v>1960</v>
+      </c>
+      <c r="I675" s="3">
+        <v>1960</v>
+      </c>
+      <c r="J675" s="3">
+        <v>7420</v>
+      </c>
+      <c r="K675" s="3">
+        <v>2402</v>
+      </c>
+      <c r="L675" s="3">
+        <v>3532</v>
+      </c>
+      <c r="M675" s="3">
+        <v>434</v>
+      </c>
+      <c r="N675" s="3">
+        <v>728</v>
+      </c>
+      <c r="O675" s="3">
+        <v>2054</v>
+      </c>
+      <c r="P675" s="3">
+        <v>9150</v>
+      </c>
+      <c r="Q675" s="4">
+        <v>89.916</v>
+      </c>
+      <c r="R675" s="4">
+        <v>0.659</v>
+      </c>
+      <c r="S675" s="4">
+        <v>6.463</v>
+      </c>
+      <c r="T675" s="4">
+        <v>0.855</v>
+      </c>
+      <c r="U675" s="4">
+        <v>0.694</v>
+      </c>
+      <c r="V675" s="4">
+        <v>0.249</v>
+      </c>
+      <c r="W675" s="4">
+        <v>1.164</v>
+      </c>
+    </row>
+    <row r="676" spans="1:23">
+      <c r="A676" s="2">
+        <v>46247</v>
+      </c>
+      <c r="B676" s="3">
+        <v>704340</v>
+      </c>
+      <c r="C676" s="3">
+        <v>3780</v>
+      </c>
+      <c r="D676" s="3">
+        <v>58520</v>
+      </c>
+      <c r="E676" s="3">
+        <v>9100</v>
+      </c>
+      <c r="F676" s="3">
+        <v>775740</v>
+      </c>
+      <c r="G676" s="3">
+        <v>3920</v>
+      </c>
+      <c r="H676" s="3">
+        <v>1960</v>
+      </c>
+      <c r="I676" s="3">
+        <v>3920</v>
+      </c>
+      <c r="J676" s="3">
+        <v>9800</v>
+      </c>
+      <c r="K676" s="3">
+        <v>2902</v>
+      </c>
+      <c r="L676" s="3">
+        <v>3198</v>
+      </c>
+      <c r="M676" s="3">
+        <v>327</v>
+      </c>
+      <c r="N676" s="3">
+        <v>623</v>
+      </c>
+      <c r="O676" s="3">
+        <v>1720</v>
+      </c>
+      <c r="P676" s="3">
+        <v>8770</v>
+      </c>
+      <c r="Q676" s="4">
+        <v>88.673</v>
+      </c>
+      <c r="R676" s="4">
+        <v>0.476</v>
+      </c>
+      <c r="S676" s="4">
+        <v>7.367</v>
+      </c>
+      <c r="T676" s="4">
+        <v>1.146</v>
+      </c>
+      <c r="U676" s="4">
+        <v>0.987</v>
+      </c>
+      <c r="V676" s="4">
+        <v>0.247</v>
+      </c>
+      <c r="W676" s="4">
+        <v>1.104</v>
+      </c>
+    </row>
+    <row r="677" spans="1:23">
+      <c r="A677" s="2">
+        <v>46248</v>
+      </c>
+      <c r="B677" s="3">
+        <v>680120</v>
+      </c>
+      <c r="C677" s="3">
+        <v>3360</v>
+      </c>
+      <c r="D677" s="3">
+        <v>74400</v>
+      </c>
+      <c r="E677" s="3">
+        <v>5180</v>
+      </c>
+      <c r="F677" s="3">
+        <v>763060</v>
+      </c>
+      <c r="G677" s="3">
+        <v>1960</v>
+      </c>
+      <c r="H677" s="3">
+        <v>1960</v>
+      </c>
+      <c r="I677" s="3">
+        <v>1960</v>
+      </c>
+      <c r="J677" s="3">
+        <v>5880</v>
+      </c>
+      <c r="K677" s="3">
+        <v>3259</v>
+      </c>
+      <c r="L677" s="3">
+        <v>3435</v>
+      </c>
+      <c r="M677" s="3">
+        <v>395</v>
+      </c>
+      <c r="N677" s="3">
+        <v>986</v>
+      </c>
+      <c r="O677" s="3">
+        <v>2360</v>
+      </c>
+      <c r="P677" s="3">
+        <v>10435</v>
+      </c>
+      <c r="Q677" s="4">
+        <v>87.265</v>
+      </c>
+      <c r="R677" s="4">
+        <v>0.431</v>
+      </c>
+      <c r="S677" s="4">
+        <v>9.546</v>
+      </c>
+      <c r="T677" s="4">
+        <v>0.665</v>
+      </c>
+      <c r="U677" s="4">
+        <v>0.503</v>
+      </c>
+      <c r="V677" s="4">
+        <v>0.251</v>
+      </c>
+      <c r="W677" s="4">
+        <v>1.339</v>
+      </c>
+    </row>
+    <row r="678" spans="1:23">
+      <c r="A678" s="2">
+        <v>46249</v>
+      </c>
+      <c r="B678" s="3">
+        <v>559300</v>
+      </c>
+      <c r="C678" s="3">
+        <v>4760</v>
+      </c>
+      <c r="D678" s="3">
+        <v>192500</v>
+      </c>
+      <c r="E678" s="3">
+        <v>5880</v>
+      </c>
+      <c r="F678" s="3">
+        <v>762440</v>
+      </c>
+      <c r="G678" s="3">
+        <v>3640</v>
+      </c>
+      <c r="H678" s="3">
+        <v>1960</v>
+      </c>
+      <c r="I678" s="3">
+        <v>0</v>
+      </c>
+      <c r="J678" s="3">
+        <v>5600</v>
+      </c>
+      <c r="K678" s="3">
+        <v>2403</v>
+      </c>
+      <c r="L678" s="3">
+        <v>3847</v>
+      </c>
+      <c r="M678" s="3">
+        <v>265</v>
+      </c>
+      <c r="N678" s="3">
+        <v>551</v>
+      </c>
+      <c r="O678" s="3">
+        <v>2267</v>
+      </c>
+      <c r="P678" s="3">
+        <v>9333</v>
+      </c>
+      <c r="Q678" s="4">
+        <v>71.947</v>
+      </c>
+      <c r="R678" s="4">
+        <v>0.612</v>
+      </c>
+      <c r="S678" s="4">
+        <v>24.763</v>
+      </c>
+      <c r="T678" s="4">
+        <v>0.756</v>
+      </c>
+      <c r="U678" s="4">
+        <v>0.468</v>
+      </c>
+      <c r="V678" s="4">
+        <v>0.252</v>
+      </c>
+      <c r="W678" s="4">
+        <v>1.201</v>
+      </c>
+    </row>
+    <row r="679" spans="1:23">
+      <c r="A679" s="2">
+        <v>46250</v>
+      </c>
+      <c r="B679" s="3">
+        <v>574980</v>
+      </c>
+      <c r="C679" s="3">
+        <v>5040</v>
+      </c>
+      <c r="D679" s="3">
+        <v>137900</v>
+      </c>
+      <c r="E679" s="3">
+        <v>5460</v>
+      </c>
+      <c r="F679" s="3">
+        <v>723380</v>
+      </c>
+      <c r="G679" s="3">
+        <v>3920</v>
+      </c>
+      <c r="H679" s="3">
+        <v>1540</v>
+      </c>
+      <c r="I679" s="3">
+        <v>0</v>
+      </c>
+      <c r="J679" s="3">
+        <v>5460</v>
+      </c>
+      <c r="K679" s="3">
+        <v>2647</v>
+      </c>
+      <c r="L679" s="3">
+        <v>3339</v>
+      </c>
+      <c r="M679" s="3">
+        <v>321</v>
+      </c>
+      <c r="N679" s="3">
+        <v>756</v>
+      </c>
+      <c r="O679" s="3">
+        <v>2141</v>
+      </c>
+      <c r="P679" s="3">
+        <v>9204</v>
+      </c>
+      <c r="Q679" s="4">
+        <v>77.906</v>
+      </c>
+      <c r="R679" s="4">
+        <v>0.683</v>
+      </c>
+      <c r="S679" s="4">
+        <v>18.685</v>
+      </c>
+      <c r="T679" s="4">
+        <v>0.740</v>
+      </c>
+      <c r="U679" s="4">
+        <v>0.531</v>
+      </c>
+      <c r="V679" s="4">
+        <v>0.209</v>
+      </c>
+      <c r="W679" s="4">
+        <v>1.247</v>
+      </c>
+    </row>
+    <row r="680" spans="1:23">
+      <c r="A680" s="2">
+        <v>46251</v>
+      </c>
+      <c r="B680" s="3">
+        <v>669480</v>
+      </c>
+      <c r="C680" s="3">
+        <v>3780</v>
+      </c>
+      <c r="D680" s="3">
+        <v>75740</v>
+      </c>
+      <c r="E680" s="3">
+        <v>3500</v>
+      </c>
+      <c r="F680" s="3">
+        <v>752500</v>
+      </c>
+      <c r="G680" s="3">
+        <v>3920</v>
+      </c>
+      <c r="H680" s="3">
+        <v>0</v>
+      </c>
+      <c r="I680" s="3">
+        <v>1960</v>
+      </c>
+      <c r="J680" s="3">
+        <v>5880</v>
+      </c>
+      <c r="K680" s="3">
+        <v>2790</v>
+      </c>
+      <c r="L680" s="3">
+        <v>4094</v>
+      </c>
+      <c r="M680" s="3">
+        <v>378</v>
+      </c>
+      <c r="N680" s="3">
+        <v>724</v>
+      </c>
+      <c r="O680" s="3">
+        <v>1961</v>
+      </c>
+      <c r="P680" s="3">
+        <v>9947</v>
+      </c>
+      <c r="Q680" s="4">
+        <v>87.135</v>
+      </c>
+      <c r="R680" s="4">
+        <v>0.492</v>
+      </c>
+      <c r="S680" s="4">
+        <v>9.858</v>
+      </c>
+      <c r="T680" s="4">
+        <v>0.456</v>
+      </c>
+      <c r="U680" s="4">
+        <v>0.765</v>
+      </c>
+      <c r="V680" s="3">
+        <v>0</v>
+      </c>
+      <c r="W680" s="4">
+        <v>1.295</v>
+      </c>
+    </row>
+    <row r="681" spans="1:23">
+      <c r="A681" s="2">
+        <v>46252</v>
+      </c>
+      <c r="B681" s="3">
+        <v>704760</v>
+      </c>
+      <c r="C681" s="3">
+        <v>5600</v>
+      </c>
+      <c r="D681" s="3">
+        <v>51800</v>
+      </c>
+      <c r="E681" s="3">
+        <v>4760</v>
+      </c>
+      <c r="F681" s="3">
+        <v>766920</v>
+      </c>
+      <c r="G681" s="3">
+        <v>1960</v>
+      </c>
+      <c r="H681" s="3">
+        <v>1960</v>
+      </c>
+      <c r="I681" s="3">
+        <v>1960</v>
+      </c>
+      <c r="J681" s="3">
+        <v>5880</v>
+      </c>
+      <c r="K681" s="3">
+        <v>2799</v>
+      </c>
+      <c r="L681" s="3">
+        <v>3955</v>
+      </c>
+      <c r="M681" s="3">
+        <v>298</v>
+      </c>
+      <c r="N681" s="3">
+        <v>720</v>
+      </c>
+      <c r="O681" s="3">
+        <v>2067</v>
+      </c>
+      <c r="P681" s="3">
+        <v>9839</v>
+      </c>
+      <c r="Q681" s="4">
+        <v>90.049</v>
+      </c>
+      <c r="R681" s="4">
+        <v>0.716</v>
+      </c>
+      <c r="S681" s="4">
+        <v>6.619</v>
+      </c>
+      <c r="T681" s="4">
+        <v>0.608</v>
+      </c>
+      <c r="U681" s="4">
+        <v>0.501</v>
+      </c>
+      <c r="V681" s="4">
+        <v>0.250</v>
+      </c>
+      <c r="W681" s="4">
+        <v>1.257</v>
+      </c>
+    </row>
+    <row r="682" spans="1:23">
+      <c r="A682" s="2">
+        <v>46253</v>
+      </c>
+      <c r="B682" s="3">
+        <v>691320</v>
+      </c>
+      <c r="C682" s="3">
+        <v>1540</v>
+      </c>
+      <c r="D682" s="3">
+        <v>45780</v>
+      </c>
+      <c r="E682" s="3">
+        <v>4900</v>
+      </c>
+      <c r="F682" s="3">
+        <v>743540</v>
+      </c>
+      <c r="G682" s="3">
+        <v>1960</v>
+      </c>
+      <c r="H682" s="3">
+        <v>1960</v>
+      </c>
+      <c r="I682" s="3">
+        <v>0</v>
+      </c>
+      <c r="J682" s="3">
+        <v>3920</v>
+      </c>
+      <c r="K682" s="3">
+        <v>2995</v>
+      </c>
+      <c r="L682" s="3">
+        <v>3756</v>
+      </c>
+      <c r="M682" s="3">
+        <v>292</v>
+      </c>
+      <c r="N682" s="3">
+        <v>615</v>
+      </c>
+      <c r="O682" s="3">
+        <v>2243</v>
+      </c>
+      <c r="P682" s="3">
+        <v>9901</v>
+      </c>
+      <c r="Q682" s="4">
+        <v>91.280</v>
+      </c>
+      <c r="R682" s="4">
+        <v>0.203</v>
+      </c>
+      <c r="S682" s="4">
+        <v>6.045</v>
+      </c>
+      <c r="T682" s="4">
+        <v>0.647</v>
+      </c>
+      <c r="U682" s="4">
+        <v>0.259</v>
+      </c>
+      <c r="V682" s="4">
+        <v>0.259</v>
+      </c>
+      <c r="W682" s="4">
+        <v>1.307</v>
+      </c>
+    </row>
+    <row r="683" spans="1:23">
+      <c r="A683" s="2">
+        <v>46254</v>
+      </c>
+      <c r="B683" s="3">
+        <v>650440</v>
+      </c>
+      <c r="C683" s="3">
+        <v>4340</v>
+      </c>
+      <c r="D683" s="3">
+        <v>35400</v>
+      </c>
+      <c r="E683" s="3">
+        <v>4900</v>
+      </c>
+      <c r="F683" s="3">
+        <v>695080</v>
+      </c>
+      <c r="G683" s="3">
+        <v>1960</v>
+      </c>
+      <c r="H683" s="3">
+        <v>1960</v>
+      </c>
+      <c r="I683" s="3">
+        <v>1960</v>
+      </c>
+      <c r="J683" s="3">
+        <v>5880</v>
+      </c>
+      <c r="K683" s="3">
+        <v>3118</v>
+      </c>
+      <c r="L683" s="3">
+        <v>3729</v>
+      </c>
+      <c r="M683" s="3">
+        <v>302</v>
+      </c>
+      <c r="N683" s="3">
+        <v>655</v>
+      </c>
+      <c r="O683" s="3">
+        <v>2547</v>
+      </c>
+      <c r="P683" s="3">
+        <v>10351</v>
+      </c>
+      <c r="Q683" s="4">
+        <v>91.442</v>
+      </c>
+      <c r="R683" s="4">
+        <v>0.610</v>
+      </c>
+      <c r="S683" s="4">
+        <v>4.977</v>
+      </c>
+      <c r="T683" s="4">
+        <v>0.689</v>
+      </c>
+      <c r="U683" s="4">
+        <v>0.551</v>
+      </c>
+      <c r="V683" s="4">
+        <v>0.276</v>
+      </c>
+      <c r="W683" s="4">
+        <v>1.455</v>
+      </c>
+    </row>
+    <row r="684" spans="1:23">
+      <c r="A684" s="2">
+        <v>46255</v>
+      </c>
+      <c r="B684" s="3">
+        <v>712040</v>
+      </c>
+      <c r="C684" s="3">
+        <v>1400</v>
+      </c>
+      <c r="D684" s="3">
+        <v>37240</v>
+      </c>
+      <c r="E684" s="3">
+        <v>4900</v>
+      </c>
+      <c r="F684" s="3">
+        <v>755580</v>
+      </c>
+      <c r="G684" s="3">
+        <v>3360</v>
+      </c>
+      <c r="H684" s="3">
+        <v>1960</v>
+      </c>
+      <c r="I684" s="3">
+        <v>1400</v>
+      </c>
+      <c r="J684" s="3">
+        <v>6720</v>
+      </c>
+      <c r="K684" s="3">
+        <v>4304</v>
+      </c>
+      <c r="L684" s="3">
+        <v>3308</v>
+      </c>
+      <c r="M684" s="3">
+        <v>341</v>
+      </c>
+      <c r="N684" s="3">
+        <v>682</v>
+      </c>
+      <c r="O684" s="3">
+        <v>2304</v>
+      </c>
+      <c r="P684" s="3">
+        <v>10939</v>
+      </c>
+      <c r="Q684" s="4">
+        <v>92.085</v>
+      </c>
+      <c r="R684" s="4">
+        <v>0.181</v>
+      </c>
+      <c r="S684" s="4">
+        <v>4.816</v>
+      </c>
+      <c r="T684" s="4">
+        <v>0.634</v>
+      </c>
+      <c r="U684" s="4">
+        <v>0.616</v>
+      </c>
+      <c r="V684" s="4">
+        <v>0.253</v>
+      </c>
+      <c r="W684" s="4">
+        <v>1.415</v>
+      </c>
+    </row>
+    <row r="685" spans="1:23">
+      <c r="A685" s="2">
+        <v>46256</v>
+      </c>
+      <c r="B685" s="3">
+        <v>679560</v>
+      </c>
+      <c r="C685" s="3">
+        <v>1400</v>
+      </c>
+      <c r="D685" s="3">
+        <v>52360</v>
+      </c>
+      <c r="E685" s="3">
+        <v>4340</v>
+      </c>
+      <c r="F685" s="3">
+        <v>737660</v>
+      </c>
+      <c r="G685" s="3">
+        <v>3500</v>
+      </c>
+      <c r="H685" s="3">
+        <v>1960</v>
+      </c>
+      <c r="I685" s="3">
+        <v>1960</v>
+      </c>
+      <c r="J685" s="3">
+        <v>7420</v>
+      </c>
+      <c r="K685" s="3">
+        <v>3371</v>
+      </c>
+      <c r="L685" s="3">
+        <v>3879</v>
+      </c>
+      <c r="M685" s="3">
+        <v>295</v>
+      </c>
+      <c r="N685" s="3">
+        <v>790</v>
+      </c>
+      <c r="O685" s="3">
+        <v>2817</v>
+      </c>
+      <c r="P685" s="3">
+        <v>11152</v>
+      </c>
+      <c r="Q685" s="4">
+        <v>89.861</v>
+      </c>
+      <c r="R685" s="4">
+        <v>0.185</v>
+      </c>
+      <c r="S685" s="4">
+        <v>6.924</v>
+      </c>
+      <c r="T685" s="4">
+        <v>0.574</v>
+      </c>
+      <c r="U685" s="4">
+        <v>0.722</v>
+      </c>
+      <c r="V685" s="4">
+        <v>0.259</v>
+      </c>
+      <c r="W685" s="4">
+        <v>1.475</v>
+      </c>
+    </row>
+    <row r="686" spans="1:23">
+      <c r="A686" s="2">
+        <v>46257</v>
+      </c>
+      <c r="B686" s="3">
+        <v>726180</v>
+      </c>
+      <c r="C686" s="3">
+        <v>5180</v>
+      </c>
+      <c r="D686" s="3">
+        <v>46760</v>
+      </c>
+      <c r="E686" s="3">
+        <v>6160</v>
+      </c>
+      <c r="F686" s="3">
+        <v>784280</v>
+      </c>
+      <c r="G686" s="3">
+        <v>3920</v>
+      </c>
+      <c r="H686" s="3">
+        <v>1960</v>
+      </c>
+      <c r="I686" s="3">
+        <v>0</v>
+      </c>
+      <c r="J686" s="3">
+        <v>5880</v>
+      </c>
+      <c r="K686" s="3">
+        <v>3156</v>
+      </c>
+      <c r="L686" s="3">
+        <v>3882</v>
+      </c>
+      <c r="M686" s="3">
+        <v>342</v>
+      </c>
+      <c r="N686" s="3">
+        <v>811</v>
+      </c>
+      <c r="O686" s="3">
+        <v>2351</v>
+      </c>
+      <c r="P686" s="3">
+        <v>10542</v>
+      </c>
+      <c r="Q686" s="4">
+        <v>90.693</v>
+      </c>
+      <c r="R686" s="4">
+        <v>0.647</v>
+      </c>
+      <c r="S686" s="4">
+        <v>5.840</v>
+      </c>
+      <c r="T686" s="4">
+        <v>0.769</v>
+      </c>
+      <c r="U686" s="4">
+        <v>0.490</v>
+      </c>
+      <c r="V686" s="4">
+        <v>0.245</v>
+      </c>
+      <c r="W686" s="4">
+        <v>1.317</v>
+      </c>
+    </row>
+    <row r="687" spans="1:23">
+      <c r="A687" s="2">
+        <v>46258</v>
+      </c>
+      <c r="B687" s="3">
+        <v>656320</v>
+      </c>
+      <c r="C687" s="3">
+        <v>1400</v>
+      </c>
+      <c r="D687" s="3">
+        <v>93800</v>
+      </c>
+      <c r="E687" s="3">
+        <v>3780</v>
+      </c>
+      <c r="F687" s="3">
+        <v>755300</v>
+      </c>
+      <c r="G687" s="3">
+        <v>3920</v>
+      </c>
+      <c r="H687" s="3">
+        <v>1960</v>
+      </c>
+      <c r="I687" s="3">
+        <v>1960</v>
+      </c>
+      <c r="J687" s="3">
+        <v>7840</v>
+      </c>
+      <c r="K687" s="3">
+        <v>3539</v>
+      </c>
+      <c r="L687" s="3">
+        <v>4287</v>
+      </c>
+      <c r="M687" s="3">
+        <v>584</v>
+      </c>
+      <c r="N687" s="3">
+        <v>762</v>
+      </c>
+      <c r="O687" s="3">
+        <v>2605</v>
+      </c>
+      <c r="P687" s="3">
+        <v>11777</v>
+      </c>
+      <c r="Q687" s="4">
+        <v>84.696</v>
+      </c>
+      <c r="R687" s="4">
+        <v>0.181</v>
+      </c>
+      <c r="S687" s="4">
+        <v>12.105</v>
+      </c>
+      <c r="T687" s="4">
+        <v>0.488</v>
+      </c>
+      <c r="U687" s="4">
+        <v>0.759</v>
+      </c>
+      <c r="V687" s="4">
+        <v>0.253</v>
+      </c>
+      <c r="W687" s="4">
+        <v>1.520</v>
+      </c>
+    </row>
+    <row r="688" spans="1:23">
+      <c r="A688" s="2">
+        <v>46259</v>
+      </c>
+      <c r="B688" s="3">
+        <v>682360</v>
+      </c>
+      <c r="C688" s="3">
+        <v>4340</v>
+      </c>
+      <c r="D688" s="3">
+        <v>95060</v>
+      </c>
+      <c r="E688" s="3">
+        <v>6300</v>
+      </c>
+      <c r="F688" s="3">
+        <v>788060</v>
+      </c>
+      <c r="G688" s="3">
+        <v>3920</v>
+      </c>
+      <c r="H688" s="3">
+        <v>1960</v>
+      </c>
+      <c r="I688" s="3">
+        <v>0</v>
+      </c>
+      <c r="J688" s="3">
+        <v>5880</v>
+      </c>
+      <c r="K688" s="3">
+        <v>3442</v>
+      </c>
+      <c r="L688" s="3">
+        <v>3886</v>
+      </c>
+      <c r="M688" s="3">
+        <v>382</v>
+      </c>
+      <c r="N688" s="3">
+        <v>593</v>
+      </c>
+      <c r="O688" s="3">
+        <v>2620</v>
+      </c>
+      <c r="P688" s="3">
+        <v>10923</v>
+      </c>
+      <c r="Q688" s="4">
+        <v>84.780</v>
+      </c>
+      <c r="R688" s="4">
+        <v>0.539</v>
+      </c>
+      <c r="S688" s="4">
+        <v>11.811</v>
+      </c>
+      <c r="T688" s="4">
+        <v>0.783</v>
+      </c>
+      <c r="U688" s="4">
+        <v>0.487</v>
+      </c>
+      <c r="V688" s="4">
+        <v>0.244</v>
+      </c>
+      <c r="W688" s="4">
+        <v>1.357</v>
+      </c>
+    </row>
+    <row r="689" spans="1:23">
+      <c r="A689" s="2">
+        <v>46260</v>
+      </c>
+      <c r="B689" s="3">
+        <v>691320</v>
+      </c>
+      <c r="C689" s="3">
+        <v>2800</v>
+      </c>
+      <c r="D689" s="3">
+        <v>64960</v>
+      </c>
+      <c r="E689" s="3">
+        <v>6440</v>
+      </c>
+      <c r="F689" s="3">
+        <v>765520</v>
+      </c>
+      <c r="G689" s="3">
+        <v>1960</v>
+      </c>
+      <c r="H689" s="3">
+        <v>1960</v>
+      </c>
+      <c r="I689" s="3">
+        <v>2940</v>
+      </c>
+      <c r="J689" s="3">
+        <v>6860</v>
+      </c>
+      <c r="K689" s="3">
+        <v>3431</v>
+      </c>
+      <c r="L689" s="3">
+        <v>3735</v>
+      </c>
+      <c r="M689" s="3">
+        <v>601</v>
+      </c>
+      <c r="N689" s="3">
+        <v>784</v>
+      </c>
+      <c r="O689" s="3">
+        <v>2992</v>
+      </c>
+      <c r="P689" s="3">
+        <v>11543</v>
+      </c>
+      <c r="Q689" s="4">
+        <v>88.187</v>
+      </c>
+      <c r="R689" s="4">
+        <v>0.357</v>
+      </c>
+      <c r="S689" s="4">
+        <v>8.287</v>
+      </c>
+      <c r="T689" s="4">
+        <v>0.822</v>
+      </c>
+      <c r="U689" s="4">
+        <v>0.625</v>
+      </c>
+      <c r="V689" s="4">
+        <v>0.250</v>
+      </c>
+      <c r="W689" s="4">
+        <v>1.472</v>
+      </c>
+    </row>
+    <row r="690" spans="1:23">
+      <c r="A690" s="2">
+        <v>46261</v>
+      </c>
+      <c r="B690" s="3">
+        <v>624820</v>
+      </c>
+      <c r="C690" s="3">
+        <v>1400</v>
+      </c>
+      <c r="D690" s="3">
+        <v>95200</v>
+      </c>
+      <c r="E690" s="3">
+        <v>6300</v>
+      </c>
+      <c r="F690" s="3">
+        <v>727720</v>
+      </c>
+      <c r="G690" s="3">
+        <v>5600</v>
+      </c>
+      <c r="H690" s="3">
+        <v>1960</v>
+      </c>
+      <c r="I690" s="3">
+        <v>0</v>
+      </c>
+      <c r="J690" s="3">
+        <v>7560</v>
+      </c>
+      <c r="K690" s="3">
+        <v>3687</v>
+      </c>
+      <c r="L690" s="3">
+        <v>5017</v>
+      </c>
+      <c r="M690" s="3">
+        <v>371</v>
+      </c>
+      <c r="N690" s="3">
+        <v>703</v>
+      </c>
+      <c r="O690" s="3">
+        <v>2488</v>
+      </c>
+      <c r="P690" s="3">
+        <v>12266</v>
+      </c>
+      <c r="Q690" s="4">
+        <v>83.583</v>
+      </c>
+      <c r="R690" s="4">
+        <v>0.187</v>
+      </c>
+      <c r="S690" s="4">
+        <v>12.735</v>
+      </c>
+      <c r="T690" s="4">
+        <v>0.843</v>
+      </c>
+      <c r="U690" s="4">
+        <v>0.749</v>
+      </c>
+      <c r="V690" s="4">
+        <v>0.262</v>
+      </c>
+      <c r="W690" s="4">
+        <v>1.641</v>
+      </c>
+    </row>
+    <row r="691" spans="1:23">
+      <c r="A691" s="2">
+        <v>46262</v>
+      </c>
+      <c r="B691" s="3">
+        <v>625380</v>
+      </c>
+      <c r="C691" s="3">
+        <v>1820</v>
+      </c>
+      <c r="D691" s="3">
+        <v>79800</v>
+      </c>
+      <c r="E691" s="3">
+        <v>9240</v>
+      </c>
+      <c r="F691" s="3">
+        <v>716240</v>
+      </c>
+      <c r="G691" s="3">
+        <v>3780</v>
+      </c>
+      <c r="H691" s="3">
+        <v>1960</v>
+      </c>
+      <c r="I691" s="3">
+        <v>1960</v>
+      </c>
+      <c r="J691" s="3">
+        <v>7700</v>
+      </c>
+      <c r="K691" s="3">
+        <v>3481</v>
+      </c>
+      <c r="L691" s="3">
+        <v>3879</v>
+      </c>
+      <c r="M691" s="3">
+        <v>413</v>
+      </c>
+      <c r="N691" s="3">
+        <v>646</v>
+      </c>
+      <c r="O691" s="3">
+        <v>2258</v>
+      </c>
+      <c r="P691" s="3">
+        <v>10677</v>
+      </c>
+      <c r="Q691" s="4">
+        <v>85.130</v>
+      </c>
+      <c r="R691" s="4">
+        <v>0.248</v>
+      </c>
+      <c r="S691" s="4">
+        <v>10.863</v>
+      </c>
+      <c r="T691" s="4">
+        <v>1.258</v>
+      </c>
+      <c r="U691" s="4">
+        <v>0.781</v>
+      </c>
+      <c r="V691" s="4">
+        <v>0.267</v>
+      </c>
+      <c r="W691" s="4">
+        <v>1.453</v>
+      </c>
+    </row>
+    <row r="692" spans="1:23">
+      <c r="A692" s="2">
+        <v>46263</v>
+      </c>
+      <c r="B692" s="3">
+        <v>694120</v>
+      </c>
+      <c r="C692" s="3">
+        <v>2940</v>
+      </c>
+      <c r="D692" s="3">
+        <v>56140</v>
+      </c>
+      <c r="E692" s="3">
+        <v>14840</v>
+      </c>
+      <c r="F692" s="3">
+        <v>768040</v>
+      </c>
+      <c r="G692" s="3">
+        <v>3920</v>
+      </c>
+      <c r="H692" s="3">
+        <v>1960</v>
+      </c>
+      <c r="I692" s="3">
+        <v>3920</v>
+      </c>
+      <c r="J692" s="3">
+        <v>9800</v>
+      </c>
+      <c r="K692" s="3">
+        <v>3257</v>
+      </c>
+      <c r="L692" s="3">
+        <v>4053</v>
+      </c>
+      <c r="M692" s="3">
+        <v>413</v>
+      </c>
+      <c r="N692" s="3">
+        <v>713</v>
+      </c>
+      <c r="O692" s="3">
+        <v>2827</v>
+      </c>
+      <c r="P692" s="3">
+        <v>11263</v>
+      </c>
+      <c r="Q692" s="4">
+        <v>87.963</v>
+      </c>
+      <c r="R692" s="4">
+        <v>0.373</v>
+      </c>
+      <c r="S692" s="4">
+        <v>7.114</v>
+      </c>
+      <c r="T692" s="4">
+        <v>1.881</v>
+      </c>
+      <c r="U692" s="4">
+        <v>0.994</v>
+      </c>
+      <c r="V692" s="4">
+        <v>0.248</v>
+      </c>
+      <c r="W692" s="4">
+        <v>1.427</v>
+      </c>
+    </row>
+    <row r="693" spans="1:23">
+      <c r="A693" s="2">
+        <v>46264</v>
+      </c>
+      <c r="B693" s="3">
+        <v>710360</v>
+      </c>
+      <c r="C693" s="3">
+        <v>3360</v>
+      </c>
+      <c r="D693" s="3">
+        <v>43680</v>
+      </c>
+      <c r="E693" s="3">
+        <v>9240</v>
+      </c>
+      <c r="F693" s="3">
+        <v>766640</v>
+      </c>
+      <c r="G693" s="3">
+        <v>3920</v>
+      </c>
+      <c r="H693" s="3">
+        <v>1960</v>
+      </c>
+      <c r="I693" s="3">
+        <v>1960</v>
+      </c>
+      <c r="J693" s="3">
+        <v>7840</v>
+      </c>
+      <c r="K693" s="3">
+        <v>3337</v>
+      </c>
+      <c r="L693" s="3">
+        <v>3333</v>
+      </c>
+      <c r="M693" s="3">
+        <v>415</v>
+      </c>
+      <c r="N693" s="3">
+        <v>809</v>
+      </c>
+      <c r="O693" s="3">
+        <v>2433</v>
+      </c>
+      <c r="P693" s="3">
+        <v>10327</v>
+      </c>
+      <c r="Q693" s="4">
+        <v>90.514</v>
+      </c>
+      <c r="R693" s="4">
+        <v>0.428</v>
+      </c>
+      <c r="S693" s="4">
+        <v>5.566</v>
+      </c>
+      <c r="T693" s="4">
+        <v>1.177</v>
+      </c>
+      <c r="U693" s="4">
+        <v>0.749</v>
+      </c>
+      <c r="V693" s="4">
+        <v>0.250</v>
+      </c>
+      <c r="W693" s="4">
+        <v>1.316</v>
+      </c>
+    </row>
+    <row r="694" spans="1:23">
+      <c r="A694" s="2">
+        <v>46265</v>
+      </c>
+      <c r="B694" s="3">
+        <v>735840</v>
+      </c>
+      <c r="C694" s="3">
+        <v>4200</v>
+      </c>
+      <c r="D694" s="3">
+        <v>31500</v>
+      </c>
+      <c r="E694" s="3">
+        <v>7280</v>
+      </c>
+      <c r="F694" s="3">
+        <v>778820</v>
+      </c>
+      <c r="G694" s="3">
+        <v>1960</v>
+      </c>
+      <c r="H694" s="3">
+        <v>3920</v>
+      </c>
+      <c r="I694" s="3">
+        <v>1960</v>
+      </c>
+      <c r="J694" s="3">
+        <v>7840</v>
+      </c>
+      <c r="K694" s="3">
+        <v>3427</v>
+      </c>
+      <c r="L694" s="3">
+        <v>3369</v>
+      </c>
+      <c r="M694" s="3">
+        <v>347</v>
+      </c>
+      <c r="N694" s="3">
+        <v>683</v>
+      </c>
+      <c r="O694" s="3">
+        <v>2362</v>
+      </c>
+      <c r="P694" s="3">
+        <v>10188</v>
+      </c>
+      <c r="Q694" s="4">
+        <v>92.344</v>
+      </c>
+      <c r="R694" s="4">
+        <v>0.527</v>
+      </c>
+      <c r="S694" s="4">
+        <v>3.953</v>
+      </c>
+      <c r="T694" s="4">
+        <v>0.914</v>
+      </c>
+      <c r="U694" s="4">
+        <v>0.492</v>
+      </c>
+      <c r="V694" s="4">
+        <v>0.492</v>
+      </c>
+      <c r="W694" s="4">
+        <v>1.279</v>
+      </c>
+    </row>
+    <row r="695" spans="1:23">
+      <c r="A695" s="2">
+        <v>46266</v>
+      </c>
+      <c r="B695" s="3">
+        <v>498960</v>
+      </c>
+      <c r="C695" s="3">
+        <v>0</v>
+      </c>
+      <c r="D695" s="3">
+        <v>21560</v>
+      </c>
+      <c r="E695" s="3">
+        <v>1960</v>
+      </c>
+      <c r="F695" s="3">
+        <v>522480</v>
+      </c>
+      <c r="G695" s="3">
+        <v>1960</v>
+      </c>
+      <c r="H695" s="3">
+        <v>0</v>
+      </c>
+      <c r="I695" s="3">
+        <v>0</v>
+      </c>
+      <c r="J695" s="3">
+        <v>1960</v>
+      </c>
+      <c r="K695" s="3">
+        <v>2653</v>
+      </c>
+      <c r="L695" s="3">
+        <v>2056</v>
+      </c>
+      <c r="M695" s="3">
+        <v>225</v>
+      </c>
+      <c r="N695" s="3">
+        <v>385</v>
+      </c>
+      <c r="O695" s="3">
+        <v>1527</v>
+      </c>
+      <c r="P695" s="3">
+        <v>6846</v>
+      </c>
+      <c r="Q695" s="4">
+        <v>93.916</v>
+      </c>
+      <c r="R695" s="3">
+        <v>0</v>
+      </c>
+      <c r="S695" s="4">
+        <v>4.058</v>
+      </c>
+      <c r="T695" s="4">
+        <v>0.369</v>
+      </c>
+      <c r="U695" s="4">
+        <v>0.369</v>
+      </c>
+      <c r="V695" s="3">
+        <v>0</v>
+      </c>
+      <c r="W695" s="4">
+        <v>1.289</v>
+      </c>
+    </row>
+    <row r="696" spans="1:23">
+      <c r="A696" s="2">
+        <v>46267</v>
+      </c>
+      <c r="B696" s="3">
+        <v>888720</v>
+      </c>
+      <c r="C696" s="3">
+        <v>7280</v>
+      </c>
+      <c r="D696" s="3">
+        <v>48860</v>
+      </c>
+      <c r="E696" s="3">
+        <v>18340</v>
+      </c>
+      <c r="F696" s="3">
+        <v>963200</v>
+      </c>
+      <c r="G696" s="3">
+        <v>5880</v>
+      </c>
+      <c r="H696" s="3">
+        <v>3780</v>
+      </c>
+      <c r="I696" s="3">
+        <v>1960</v>
+      </c>
+      <c r="J696" s="3">
+        <v>11620</v>
+      </c>
+      <c r="K696" s="3">
+        <v>5081</v>
+      </c>
+      <c r="L696" s="3">
+        <v>4845</v>
+      </c>
+      <c r="M696" s="3">
+        <v>638</v>
+      </c>
+      <c r="N696" s="3">
+        <v>1195</v>
+      </c>
+      <c r="O696" s="3">
+        <v>3568</v>
+      </c>
+      <c r="P696" s="3">
+        <v>15327</v>
+      </c>
+      <c r="Q696" s="4">
+        <v>89.756</v>
+      </c>
+      <c r="R696" s="4">
+        <v>0.735</v>
+      </c>
+      <c r="S696" s="4">
+        <v>4.935</v>
+      </c>
+      <c r="T696" s="4">
+        <v>1.852</v>
+      </c>
+      <c r="U696" s="4">
+        <v>0.792</v>
+      </c>
+      <c r="V696" s="4">
+        <v>0.382</v>
+      </c>
+      <c r="W696" s="4">
+        <v>1.548</v>
+      </c>
+    </row>
+    <row r="697" spans="1:23">
+      <c r="A697" s="2">
+        <v>46268</v>
+      </c>
+      <c r="B697" s="3">
+        <v>690760</v>
+      </c>
+      <c r="C697" s="3">
+        <v>0</v>
+      </c>
+      <c r="D697" s="3">
+        <v>29400</v>
+      </c>
+      <c r="E697" s="3">
+        <v>7420</v>
+      </c>
+      <c r="F697" s="3">
+        <v>727580</v>
+      </c>
+      <c r="G697" s="3">
+        <v>4260</v>
+      </c>
+      <c r="H697" s="3">
+        <v>1820</v>
+      </c>
+      <c r="I697" s="3">
+        <v>1960</v>
+      </c>
+      <c r="J697" s="3">
+        <v>8040</v>
+      </c>
+      <c r="K697" s="3">
+        <v>3865</v>
+      </c>
+      <c r="L697" s="3">
+        <v>4095</v>
+      </c>
+      <c r="M697" s="3">
+        <v>317</v>
+      </c>
+      <c r="N697" s="3">
+        <v>881</v>
+      </c>
+      <c r="O697" s="3">
+        <v>2448</v>
+      </c>
+      <c r="P697" s="3">
+        <v>11606</v>
+      </c>
+      <c r="Q697" s="4">
+        <v>92.443</v>
+      </c>
+      <c r="R697" s="3">
+        <v>0</v>
+      </c>
+      <c r="S697" s="4">
+        <v>3.935</v>
+      </c>
+      <c r="T697" s="4">
+        <v>0.993</v>
+      </c>
+      <c r="U697" s="4">
+        <v>0.832</v>
+      </c>
+      <c r="V697" s="4">
+        <v>0.244</v>
+      </c>
+      <c r="W697" s="4">
+        <v>1.553</v>
+      </c>
+    </row>
+    <row r="698" spans="1:23">
+      <c r="A698" s="2">
+        <v>46269</v>
+      </c>
+      <c r="B698" s="3">
+        <v>745360</v>
+      </c>
+      <c r="C698" s="3">
+        <v>6440</v>
+      </c>
+      <c r="D698" s="3">
+        <v>22120</v>
+      </c>
+      <c r="E698" s="3">
+        <v>3360</v>
+      </c>
+      <c r="F698" s="3">
+        <v>777280</v>
+      </c>
+      <c r="G698" s="3">
+        <v>3920</v>
+      </c>
+      <c r="H698" s="3">
+        <v>1680</v>
+      </c>
+      <c r="I698" s="3">
+        <v>1960</v>
+      </c>
+      <c r="J698" s="3">
+        <v>7560</v>
+      </c>
+      <c r="K698" s="3">
+        <v>2721</v>
+      </c>
+      <c r="L698" s="3">
+        <v>3956</v>
+      </c>
+      <c r="M698" s="3">
+        <v>300</v>
+      </c>
+      <c r="N698" s="3">
+        <v>742</v>
+      </c>
+      <c r="O698" s="3">
+        <v>2510</v>
+      </c>
+      <c r="P698" s="3">
+        <v>10229</v>
+      </c>
+      <c r="Q698" s="4">
+        <v>93.748</v>
+      </c>
+      <c r="R698" s="4">
+        <v>0.810</v>
+      </c>
+      <c r="S698" s="4">
+        <v>2.782</v>
+      </c>
+      <c r="T698" s="4">
+        <v>0.423</v>
+      </c>
+      <c r="U698" s="4">
+        <v>0.740</v>
+      </c>
+      <c r="V698" s="4">
+        <v>0.211</v>
+      </c>
+      <c r="W698" s="4">
+        <v>1.287</v>
+      </c>
+    </row>
+    <row r="699" spans="1:23">
+      <c r="A699" s="2">
+        <v>46270</v>
+      </c>
+      <c r="B699" s="3">
+        <v>690200</v>
+      </c>
+      <c r="C699" s="3">
+        <v>4340</v>
+      </c>
+      <c r="D699" s="3">
+        <v>29960</v>
+      </c>
+      <c r="E699" s="3">
+        <v>7840</v>
+      </c>
+      <c r="F699" s="3">
+        <v>732340</v>
+      </c>
+      <c r="G699" s="3">
+        <v>3920</v>
+      </c>
+      <c r="H699" s="3">
+        <v>1540</v>
+      </c>
+      <c r="I699" s="3">
+        <v>1960</v>
+      </c>
+      <c r="J699" s="3">
+        <v>7420</v>
+      </c>
+      <c r="K699" s="3">
+        <v>3475</v>
+      </c>
+      <c r="L699" s="3">
+        <v>4149</v>
+      </c>
+      <c r="M699" s="3">
+        <v>355</v>
+      </c>
+      <c r="N699" s="3">
+        <v>770</v>
+      </c>
+      <c r="O699" s="3">
+        <v>2553</v>
+      </c>
+      <c r="P699" s="3">
+        <v>11302</v>
+      </c>
+      <c r="Q699" s="4">
+        <v>91.897</v>
+      </c>
+      <c r="R699" s="4">
+        <v>0.578</v>
+      </c>
+      <c r="S699" s="4">
+        <v>3.989</v>
+      </c>
+      <c r="T699" s="4">
+        <v>1.044</v>
+      </c>
+      <c r="U699" s="4">
+        <v>0.783</v>
+      </c>
+      <c r="V699" s="4">
+        <v>0.205</v>
+      </c>
+      <c r="W699" s="4">
+        <v>1.505</v>
+      </c>
+    </row>
+    <row r="700" spans="1:23">
+      <c r="A700" s="2">
+        <v>46271</v>
+      </c>
+      <c r="B700" s="3">
+        <v>712320</v>
+      </c>
+      <c r="C700" s="3">
+        <v>5040</v>
+      </c>
+      <c r="D700" s="3">
+        <v>50820</v>
+      </c>
+      <c r="E700" s="3">
+        <v>6720</v>
+      </c>
+      <c r="F700" s="3">
+        <v>774900</v>
+      </c>
+      <c r="G700" s="3">
+        <v>3920</v>
+      </c>
+      <c r="H700" s="3">
+        <v>1680</v>
+      </c>
+      <c r="I700" s="3">
+        <v>1680</v>
+      </c>
+      <c r="J700" s="3">
+        <v>7280</v>
+      </c>
+      <c r="K700" s="3">
+        <v>2755</v>
+      </c>
+      <c r="L700" s="3">
+        <v>3686</v>
+      </c>
+      <c r="M700" s="3">
+        <v>367</v>
+      </c>
+      <c r="N700" s="3">
+        <v>838</v>
+      </c>
+      <c r="O700" s="3">
+        <v>2841</v>
+      </c>
+      <c r="P700" s="3">
+        <v>10487</v>
+      </c>
+      <c r="Q700" s="4">
+        <v>89.864</v>
+      </c>
+      <c r="R700" s="4">
+        <v>0.636</v>
+      </c>
+      <c r="S700" s="4">
+        <v>6.411</v>
+      </c>
+      <c r="T700" s="4">
+        <v>0.848</v>
+      </c>
+      <c r="U700" s="4">
+        <v>0.706</v>
+      </c>
+      <c r="V700" s="4">
+        <v>0.212</v>
+      </c>
+      <c r="W700" s="4">
+        <v>1.323</v>
+      </c>
+    </row>
+    <row r="701" spans="1:23">
+      <c r="A701" s="2">
+        <v>46272</v>
+      </c>
+      <c r="B701" s="3">
+        <v>703080</v>
+      </c>
+      <c r="C701" s="3">
+        <v>1960</v>
+      </c>
+      <c r="D701" s="3">
+        <v>54180</v>
+      </c>
+      <c r="E701" s="3">
+        <v>9100</v>
+      </c>
+      <c r="F701" s="3">
+        <v>768320</v>
+      </c>
+      <c r="G701" s="3">
+        <v>5880</v>
+      </c>
+      <c r="H701" s="3">
+        <v>1960</v>
+      </c>
+      <c r="I701" s="3">
+        <v>1960</v>
+      </c>
+      <c r="J701" s="3">
+        <v>9800</v>
+      </c>
+      <c r="K701" s="3">
+        <v>2765</v>
+      </c>
+      <c r="L701" s="3">
+        <v>3964</v>
+      </c>
+      <c r="M701" s="3">
+        <v>322</v>
+      </c>
+      <c r="N701" s="3">
+        <v>787</v>
+      </c>
+      <c r="O701" s="3">
+        <v>2612</v>
+      </c>
+      <c r="P701" s="3">
+        <v>10450</v>
+      </c>
+      <c r="Q701" s="4">
+        <v>89.159</v>
+      </c>
+      <c r="R701" s="4">
+        <v>0.249</v>
+      </c>
+      <c r="S701" s="4">
+        <v>6.871</v>
+      </c>
+      <c r="T701" s="4">
+        <v>1.154</v>
+      </c>
+      <c r="U701" s="4">
+        <v>0.994</v>
+      </c>
+      <c r="V701" s="4">
+        <v>0.249</v>
+      </c>
+      <c r="W701" s="4">
+        <v>1.325</v>
+      </c>
+    </row>
+    <row r="702" spans="1:23">
+      <c r="A702" s="2">
+        <v>46273</v>
+      </c>
+      <c r="B702" s="3">
+        <v>698040</v>
+      </c>
+      <c r="C702" s="3">
+        <v>1960</v>
+      </c>
+      <c r="D702" s="3">
+        <v>70840</v>
+      </c>
+      <c r="E702" s="3">
+        <v>8120</v>
+      </c>
+      <c r="F702" s="3">
+        <v>778960</v>
+      </c>
+      <c r="G702" s="3">
+        <v>3920</v>
+      </c>
+      <c r="H702" s="3">
+        <v>1960</v>
+      </c>
+      <c r="I702" s="3">
+        <v>1960</v>
+      </c>
+      <c r="J702" s="3">
+        <v>7840</v>
+      </c>
+      <c r="K702" s="3">
+        <v>3008</v>
+      </c>
+      <c r="L702" s="3">
+        <v>2948</v>
+      </c>
+      <c r="M702" s="3">
+        <v>291</v>
+      </c>
+      <c r="N702" s="3">
+        <v>691</v>
+      </c>
+      <c r="O702" s="3">
+        <v>2374</v>
+      </c>
+      <c r="P702" s="3">
+        <v>9312</v>
+      </c>
+      <c r="Q702" s="4">
+        <v>87.681</v>
+      </c>
+      <c r="R702" s="4">
+        <v>0.246</v>
+      </c>
+      <c r="S702" s="4">
+        <v>8.898</v>
+      </c>
+      <c r="T702" s="4">
+        <v>1.020</v>
+      </c>
+      <c r="U702" s="4">
+        <v>0.739</v>
+      </c>
+      <c r="V702" s="4">
+        <v>0.246</v>
+      </c>
+      <c r="W702" s="4">
+        <v>1.170</v>
+      </c>
+    </row>
+    <row r="703" spans="1:23">
+      <c r="A703" s="2">
+        <v>46274</v>
+      </c>
+      <c r="B703" s="3">
+        <v>651840</v>
+      </c>
+      <c r="C703" s="3">
+        <v>7840</v>
+      </c>
+      <c r="D703" s="3">
+        <v>66500</v>
+      </c>
+      <c r="E703" s="3">
+        <v>6440</v>
+      </c>
+      <c r="F703" s="3">
+        <v>732620</v>
+      </c>
+      <c r="G703" s="3">
+        <v>5880</v>
+      </c>
+      <c r="H703" s="3">
+        <v>1960</v>
+      </c>
+      <c r="I703" s="3">
+        <v>1960</v>
+      </c>
+      <c r="J703" s="3">
+        <v>9800</v>
+      </c>
+      <c r="K703" s="3">
+        <v>4661</v>
+      </c>
+      <c r="L703" s="3">
+        <v>2850</v>
+      </c>
+      <c r="M703" s="3">
+        <v>606</v>
+      </c>
+      <c r="N703" s="3">
+        <v>760</v>
+      </c>
+      <c r="O703" s="3">
+        <v>2572</v>
+      </c>
+      <c r="P703" s="3">
+        <v>11449</v>
+      </c>
+      <c r="Q703" s="4">
+        <v>86.466</v>
+      </c>
+      <c r="R703" s="4">
+        <v>1.040</v>
+      </c>
+      <c r="S703" s="4">
+        <v>8.821</v>
+      </c>
+      <c r="T703" s="4">
+        <v>0.854</v>
+      </c>
+      <c r="U703" s="4">
+        <v>1.040</v>
+      </c>
+      <c r="V703" s="4">
+        <v>0.260</v>
+      </c>
+      <c r="W703" s="4">
+        <v>1.519</v>
+      </c>
+    </row>
+    <row r="704" spans="1:23">
+      <c r="A704" s="2">
+        <v>46275</v>
+      </c>
+      <c r="B704" s="3">
+        <v>574840</v>
+      </c>
+      <c r="C704" s="3">
+        <v>5880</v>
+      </c>
+      <c r="D704" s="3">
+        <v>178500</v>
+      </c>
+      <c r="E704" s="3">
+        <v>9660</v>
+      </c>
+      <c r="F704" s="3">
+        <v>768880</v>
+      </c>
+      <c r="G704" s="3">
+        <v>3920</v>
+      </c>
+      <c r="H704" s="3">
+        <v>1960</v>
+      </c>
+      <c r="I704" s="3">
+        <v>1960</v>
+      </c>
+      <c r="J704" s="3">
+        <v>7840</v>
+      </c>
+      <c r="K704" s="3">
+        <v>3211</v>
+      </c>
+      <c r="L704" s="3">
+        <v>2449</v>
+      </c>
+      <c r="M704" s="3">
+        <v>448</v>
+      </c>
+      <c r="N704" s="3">
+        <v>747</v>
+      </c>
+      <c r="O704" s="3">
+        <v>2454</v>
+      </c>
+      <c r="P704" s="3">
+        <v>9309</v>
+      </c>
+      <c r="Q704" s="4">
+        <v>73.132</v>
+      </c>
+      <c r="R704" s="4">
+        <v>0.748</v>
+      </c>
+      <c r="S704" s="4">
+        <v>22.709</v>
+      </c>
+      <c r="T704" s="4">
+        <v>1.229</v>
+      </c>
+      <c r="U704" s="4">
+        <v>0.748</v>
+      </c>
+      <c r="V704" s="4">
+        <v>0.249</v>
+      </c>
+      <c r="W704" s="4">
+        <v>1.184</v>
+      </c>
+    </row>
+    <row r="705" spans="1:23">
+      <c r="A705" s="2">
+        <v>46276</v>
+      </c>
+      <c r="B705" s="3">
+        <v>425040</v>
+      </c>
+      <c r="C705" s="3">
+        <v>5880</v>
+      </c>
+      <c r="D705" s="3">
+        <v>109060</v>
+      </c>
+      <c r="E705" s="3">
+        <v>7000</v>
+      </c>
+      <c r="F705" s="3">
+        <v>546980</v>
+      </c>
+      <c r="G705" s="3">
+        <v>5880</v>
+      </c>
+      <c r="H705" s="3">
+        <v>1960</v>
+      </c>
+      <c r="I705" s="3">
+        <v>0</v>
+      </c>
+      <c r="J705" s="3">
+        <v>7840</v>
+      </c>
+      <c r="K705" s="3">
+        <v>2430</v>
+      </c>
+      <c r="L705" s="3">
+        <v>2603</v>
+      </c>
+      <c r="M705" s="3">
+        <v>428</v>
+      </c>
+      <c r="N705" s="3">
+        <v>785</v>
+      </c>
+      <c r="O705" s="3">
+        <v>1986</v>
+      </c>
+      <c r="P705" s="3">
+        <v>8232</v>
+      </c>
+      <c r="Q705" s="4">
+        <v>75.489</v>
+      </c>
+      <c r="R705" s="4">
+        <v>1.044</v>
+      </c>
+      <c r="S705" s="4">
+        <v>19.369</v>
+      </c>
+      <c r="T705" s="4">
+        <v>1.243</v>
+      </c>
+      <c r="U705" s="4">
+        <v>1.044</v>
+      </c>
+      <c r="V705" s="4">
+        <v>0.348</v>
+      </c>
+      <c r="W705" s="4">
+        <v>1.462</v>
+      </c>
+    </row>
+    <row r="706" spans="1:23">
+      <c r="A706" s="2">
+        <v>46277</v>
+      </c>
+      <c r="B706" s="3">
+        <v>554960</v>
+      </c>
+      <c r="C706" s="3">
+        <v>5320</v>
+      </c>
+      <c r="D706" s="3">
+        <v>113540</v>
+      </c>
+      <c r="E706" s="3">
+        <v>11620</v>
+      </c>
+      <c r="F706" s="3">
+        <v>685440</v>
+      </c>
+      <c r="G706" s="3">
+        <v>3920</v>
+      </c>
+      <c r="H706" s="3">
+        <v>1960</v>
+      </c>
+      <c r="I706" s="3">
+        <v>3920</v>
+      </c>
+      <c r="J706" s="3">
+        <v>9800</v>
+      </c>
+      <c r="K706" s="3">
+        <v>2956</v>
+      </c>
+      <c r="L706" s="3">
+        <v>3494</v>
+      </c>
+      <c r="M706" s="3">
+        <v>368</v>
+      </c>
+      <c r="N706" s="3">
+        <v>914</v>
+      </c>
+      <c r="O706" s="3">
+        <v>2469</v>
+      </c>
+      <c r="P706" s="3">
+        <v>10201</v>
+      </c>
+      <c r="Q706" s="4">
+        <v>78.669</v>
+      </c>
+      <c r="R706" s="4">
+        <v>0.754</v>
+      </c>
+      <c r="S706" s="4">
+        <v>16.095</v>
+      </c>
+      <c r="T706" s="4">
+        <v>1.647</v>
+      </c>
+      <c r="U706" s="4">
+        <v>1.111</v>
+      </c>
+      <c r="V706" s="4">
+        <v>0.278</v>
+      </c>
+      <c r="W706" s="4">
+        <v>1.446</v>
+      </c>
+    </row>
+    <row r="707" spans="1:23">
+      <c r="A707" s="2">
+        <v>46278</v>
+      </c>
+      <c r="B707" s="3">
+        <v>611240</v>
+      </c>
+      <c r="C707" s="3">
+        <v>10780</v>
+      </c>
+      <c r="D707" s="3">
+        <v>93380</v>
+      </c>
+      <c r="E707" s="3">
+        <v>7560</v>
+      </c>
+      <c r="F707" s="3">
+        <v>722960</v>
+      </c>
+      <c r="G707" s="3">
+        <v>7840</v>
+      </c>
+      <c r="H707" s="3">
+        <v>1960</v>
+      </c>
+      <c r="I707" s="3">
+        <v>0</v>
+      </c>
+      <c r="J707" s="3">
+        <v>9800</v>
+      </c>
+      <c r="K707" s="3">
+        <v>2945</v>
+      </c>
+      <c r="L707" s="3">
+        <v>3714</v>
+      </c>
+      <c r="M707" s="3">
+        <v>428</v>
+      </c>
+      <c r="N707" s="3">
+        <v>859</v>
+      </c>
+      <c r="O707" s="3">
+        <v>2329</v>
+      </c>
+      <c r="P707" s="3">
+        <v>10275</v>
+      </c>
+      <c r="Q707" s="4">
+        <v>82.263</v>
+      </c>
+      <c r="R707" s="4">
+        <v>1.451</v>
+      </c>
+      <c r="S707" s="4">
+        <v>12.567</v>
+      </c>
+      <c r="T707" s="4">
+        <v>1.017</v>
+      </c>
+      <c r="U707" s="4">
+        <v>1.055</v>
+      </c>
+      <c r="V707" s="4">
+        <v>0.264</v>
+      </c>
+      <c r="W707" s="4">
+        <v>1.383</v>
+      </c>
+    </row>
+    <row r="708" spans="1:23">
+      <c r="A708" s="2">
+        <v>46279</v>
+      </c>
+      <c r="B708" s="3">
+        <v>708680</v>
+      </c>
+      <c r="C708" s="3">
+        <v>1960</v>
+      </c>
+      <c r="D708" s="3">
+        <v>31920</v>
+      </c>
+      <c r="E708" s="3">
+        <v>0</v>
+      </c>
+      <c r="F708" s="3">
+        <v>742560</v>
+      </c>
+      <c r="G708" s="3">
+        <v>3920</v>
+      </c>
+      <c r="H708" s="3">
+        <v>1960</v>
+      </c>
+      <c r="I708" s="3">
+        <v>1960</v>
+      </c>
+      <c r="J708" s="3">
+        <v>7840</v>
+      </c>
+      <c r="K708" s="3">
+        <v>3077</v>
+      </c>
+      <c r="L708" s="3">
+        <v>2983</v>
+      </c>
+      <c r="M708" s="3">
+        <v>450</v>
+      </c>
+      <c r="N708" s="3">
+        <v>857</v>
+      </c>
+      <c r="O708" s="3">
+        <v>2401</v>
+      </c>
+      <c r="P708" s="3">
+        <v>9768</v>
+      </c>
+      <c r="Q708" s="4">
+        <v>93.227</v>
+      </c>
+      <c r="R708" s="4">
+        <v>0.258</v>
+      </c>
+      <c r="S708" s="4">
+        <v>4.199</v>
+      </c>
+      <c r="T708" s="3">
+        <v>0</v>
+      </c>
+      <c r="U708" s="4">
+        <v>0.774</v>
+      </c>
+      <c r="V708" s="4">
+        <v>0.258</v>
+      </c>
+      <c r="W708" s="4">
+        <v>1.285</v>
+      </c>
+    </row>
+    <row r="709" spans="1:23">
+      <c r="A709" s="2">
+        <v>46280</v>
+      </c>
+      <c r="B709" s="3">
+        <v>654080</v>
+      </c>
+      <c r="C709" s="3">
+        <v>9660</v>
+      </c>
+      <c r="D709" s="3">
+        <v>17080</v>
+      </c>
+      <c r="E709" s="3">
+        <v>15680</v>
+      </c>
+      <c r="F709" s="3">
+        <v>696500</v>
+      </c>
+      <c r="G709" s="3">
+        <v>1960</v>
+      </c>
+      <c r="H709" s="3">
+        <v>1960</v>
+      </c>
+      <c r="I709" s="3">
+        <v>1960</v>
+      </c>
+      <c r="J709" s="3">
+        <v>5880</v>
+      </c>
+      <c r="K709" s="3">
+        <v>2561</v>
+      </c>
+      <c r="L709" s="3">
+        <v>3124</v>
+      </c>
+      <c r="M709" s="3">
+        <v>320</v>
+      </c>
+      <c r="N709" s="3">
+        <v>728</v>
+      </c>
+      <c r="O709" s="3">
+        <v>2026</v>
+      </c>
+      <c r="P709" s="3">
+        <v>8759</v>
+      </c>
+      <c r="Q709" s="4">
+        <v>91.976</v>
+      </c>
+      <c r="R709" s="4">
+        <v>1.358</v>
+      </c>
+      <c r="S709" s="4">
+        <v>2.402</v>
+      </c>
+      <c r="T709" s="4">
+        <v>2.205</v>
+      </c>
+      <c r="U709" s="4">
+        <v>0.551</v>
+      </c>
+      <c r="V709" s="4">
+        <v>0.276</v>
+      </c>
+      <c r="W709" s="4">
+        <v>1.232</v>
+      </c>
+    </row>
+    <row r="710" spans="1:23">
+      <c r="A710" s="2">
+        <v>46281</v>
+      </c>
+      <c r="B710" s="3">
+        <v>636800</v>
+      </c>
+      <c r="C710" s="3">
+        <v>5460</v>
+      </c>
+      <c r="D710" s="3">
+        <v>24640</v>
+      </c>
+      <c r="E710" s="3">
+        <v>3080</v>
+      </c>
+      <c r="F710" s="3">
+        <v>669980</v>
+      </c>
+      <c r="G710" s="3">
+        <v>1960</v>
+      </c>
+      <c r="H710" s="3">
+        <v>1960</v>
+      </c>
+      <c r="I710" s="3">
+        <v>1960</v>
+      </c>
+      <c r="J710" s="3">
+        <v>5880</v>
+      </c>
+      <c r="K710" s="3">
+        <v>3082</v>
+      </c>
+      <c r="L710" s="3">
+        <v>3627</v>
+      </c>
+      <c r="M710" s="3">
+        <v>394</v>
+      </c>
+      <c r="N710" s="3">
+        <v>818</v>
+      </c>
+      <c r="O710" s="3">
+        <v>1896</v>
+      </c>
+      <c r="P710" s="3">
+        <v>9817</v>
+      </c>
+      <c r="Q710" s="4">
+        <v>92.872</v>
+      </c>
+      <c r="R710" s="4">
+        <v>0.796</v>
+      </c>
+      <c r="S710" s="4">
+        <v>3.594</v>
+      </c>
+      <c r="T710" s="4">
+        <v>0.449</v>
+      </c>
+      <c r="U710" s="4">
+        <v>0.572</v>
+      </c>
+      <c r="V710" s="4">
+        <v>0.286</v>
+      </c>
+      <c r="W710" s="4">
+        <v>1.432</v>
+      </c>
+    </row>
+    <row r="711" spans="1:23">
+      <c r="A711" s="2">
+        <v>46282</v>
+      </c>
+      <c r="B711" s="3">
+        <v>520560</v>
+      </c>
+      <c r="C711" s="3">
+        <v>8260</v>
+      </c>
+      <c r="D711" s="3">
+        <v>34440</v>
+      </c>
+      <c r="E711" s="3">
+        <v>2940</v>
+      </c>
+      <c r="F711" s="3">
+        <v>566200</v>
+      </c>
+      <c r="G711" s="3">
+        <v>3920</v>
+      </c>
+      <c r="H711" s="3">
+        <v>3920</v>
+      </c>
+      <c r="I711" s="3">
+        <v>1960</v>
+      </c>
+      <c r="J711" s="3">
+        <v>9800</v>
+      </c>
+      <c r="K711" s="3">
+        <v>4262</v>
+      </c>
+      <c r="L711" s="3">
+        <v>3442</v>
+      </c>
+      <c r="M711" s="3">
+        <v>294</v>
+      </c>
+      <c r="N711" s="3">
+        <v>1463</v>
+      </c>
+      <c r="O711" s="3">
+        <v>1955</v>
+      </c>
+      <c r="P711" s="3">
+        <v>11416</v>
+      </c>
+      <c r="Q711" s="4">
+        <v>88.619</v>
+      </c>
+      <c r="R711" s="4">
+        <v>1.406</v>
+      </c>
+      <c r="S711" s="4">
+        <v>5.863</v>
+      </c>
+      <c r="T711" s="4">
+        <v>0.500</v>
+      </c>
+      <c r="U711" s="4">
+        <v>1.001</v>
+      </c>
+      <c r="V711" s="4">
+        <v>0.667</v>
+      </c>
+      <c r="W711" s="4">
+        <v>1.943</v>
+      </c>
+    </row>
+    <row r="712" spans="1:23">
+      <c r="A712" s="2">
+        <v>46283</v>
+      </c>
+      <c r="B712" s="3">
+        <v>575680</v>
+      </c>
+      <c r="C712" s="3">
+        <v>5600</v>
+      </c>
+      <c r="D712" s="3">
+        <v>34020</v>
+      </c>
+      <c r="E712" s="3">
+        <v>1960</v>
+      </c>
+      <c r="F712" s="3">
+        <v>617260</v>
+      </c>
+      <c r="G712" s="3">
+        <v>9800</v>
+      </c>
+      <c r="H712" s="3">
+        <v>1960</v>
+      </c>
+      <c r="I712" s="3">
+        <v>1960</v>
+      </c>
+      <c r="J712" s="3">
+        <v>13720</v>
+      </c>
+      <c r="K712" s="3">
+        <v>4071</v>
+      </c>
+      <c r="L712" s="3">
+        <v>4386</v>
+      </c>
+      <c r="M712" s="3">
+        <v>403</v>
+      </c>
+      <c r="N712" s="3">
+        <v>1135</v>
+      </c>
+      <c r="O712" s="3">
+        <v>2168</v>
+      </c>
+      <c r="P712" s="3">
+        <v>12163</v>
+      </c>
+      <c r="Q712" s="4">
+        <v>89.510</v>
+      </c>
+      <c r="R712" s="4">
+        <v>0.871</v>
+      </c>
+      <c r="S712" s="4">
+        <v>5.290</v>
+      </c>
+      <c r="T712" s="4">
+        <v>0.305</v>
+      </c>
+      <c r="U712" s="4">
+        <v>1.829</v>
+      </c>
+      <c r="V712" s="4">
+        <v>0.305</v>
+      </c>
+      <c r="W712" s="4">
+        <v>1.891</v>
+      </c>
+    </row>
+    <row r="713" spans="1:23">
+      <c r="A713" s="2">
+        <v>46284</v>
+      </c>
+      <c r="B713" s="3">
+        <v>302960</v>
+      </c>
+      <c r="C713" s="3">
+        <v>0</v>
+      </c>
+      <c r="D713" s="3">
+        <v>9800</v>
+      </c>
+      <c r="E713" s="3">
+        <v>1960</v>
+      </c>
+      <c r="F713" s="3">
+        <v>314720</v>
+      </c>
+      <c r="G713" s="3">
+        <v>1960</v>
+      </c>
+      <c r="H713" s="3">
+        <v>0</v>
+      </c>
+      <c r="I713" s="3">
+        <v>1960</v>
+      </c>
+      <c r="J713" s="3">
+        <v>3920</v>
+      </c>
+      <c r="K713" s="3">
+        <v>1320</v>
+      </c>
+      <c r="L713" s="3">
+        <v>1176</v>
+      </c>
+      <c r="M713" s="3">
+        <v>104</v>
+      </c>
+      <c r="N713" s="3">
+        <v>213</v>
+      </c>
+      <c r="O713" s="3">
+        <v>641</v>
+      </c>
+      <c r="P713" s="3">
+        <v>3454</v>
+      </c>
+      <c r="Q713" s="4">
+        <v>94.059</v>
+      </c>
+      <c r="R713" s="3">
+        <v>0</v>
+      </c>
+      <c r="S713" s="4">
+        <v>3.043</v>
+      </c>
+      <c r="T713" s="4">
+        <v>0.609</v>
+      </c>
+      <c r="U713" s="4">
+        <v>1.217</v>
+      </c>
+      <c r="V713" s="3">
+        <v>0</v>
+      </c>
+      <c r="W713" s="4">
+        <v>1.072</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sync latest local data and SAP script updates
</commit_message>
<xml_diff>
--- a/backend/data/Daywise Data.xlsx
+++ b/backend/data/Daywise Data.xlsx
@@ -1373,10 +1373,10 @@
         <v>87360</v>
       </c>
       <c r="G17" s="3">
-        <v>0</v>
+        <v>1440</v>
       </c>
       <c r="H17" s="3">
-        <v>1440</v>
+        <v>0</v>
       </c>
       <c r="I17" s="3">
         <v>0</v>
@@ -1414,11 +1414,11 @@
       <c r="T17" s="3">
         <v>0</v>
       </c>
-      <c r="U17" s="3">
-        <v>0</v>
-      </c>
-      <c r="V17" s="4">
+      <c r="U17" s="4">
         <v>1.572</v>
+      </c>
+      <c r="V17" s="3">
+        <v>0</v>
       </c>
       <c r="W17" s="4">
         <v>3.031</v>
@@ -1713,13 +1713,13 @@
         <v>45591</v>
       </c>
       <c r="B22" s="3">
-        <v>6720</v>
+        <v>8040</v>
       </c>
       <c r="C22" s="3">
         <v>0</v>
       </c>
       <c r="D22" s="3">
-        <v>65880</v>
+        <v>64560</v>
       </c>
       <c r="E22" s="3">
         <v>1680</v>
@@ -1758,13 +1758,13 @@
         <v>1620</v>
       </c>
       <c r="Q22" s="4">
-        <v>8.757</v>
+        <v>10.477</v>
       </c>
       <c r="R22" s="3">
         <v>0</v>
       </c>
       <c r="S22" s="4">
-        <v>85.848</v>
+        <v>84.128</v>
       </c>
       <c r="T22" s="4">
         <v>2.189</v>
@@ -1855,13 +1855,13 @@
         <v>45593</v>
       </c>
       <c r="B24" s="3">
-        <v>12480</v>
+        <v>14160</v>
       </c>
       <c r="C24" s="3">
         <v>10560</v>
       </c>
       <c r="D24" s="3">
-        <v>101400</v>
+        <v>99720</v>
       </c>
       <c r="E24" s="3">
         <v>3360</v>
@@ -1900,13 +1900,13 @@
         <v>1978</v>
       </c>
       <c r="Q24" s="4">
-        <v>9.273</v>
+        <v>10.522</v>
       </c>
       <c r="R24" s="4">
         <v>7.847</v>
       </c>
       <c r="S24" s="4">
-        <v>75.347</v>
+        <v>74.098</v>
       </c>
       <c r="T24" s="4">
         <v>2.497</v>
@@ -3488,13 +3488,13 @@
         <v>45616</v>
       </c>
       <c r="B47" s="3">
-        <v>182880</v>
+        <v>181200</v>
       </c>
       <c r="C47" s="3">
         <v>1560</v>
       </c>
       <c r="D47" s="3">
-        <v>73200</v>
+        <v>74880</v>
       </c>
       <c r="E47" s="3">
         <v>0</v>
@@ -3533,13 +3533,13 @@
         <v>3636</v>
       </c>
       <c r="Q47" s="4">
-        <v>69.995</v>
+        <v>69.352</v>
       </c>
       <c r="R47" s="4">
         <v>0.597</v>
       </c>
       <c r="S47" s="4">
-        <v>28.016</v>
+        <v>28.659</v>
       </c>
       <c r="T47" s="3">
         <v>0</v>
@@ -50774,19 +50774,19 @@
         <v>46284</v>
       </c>
       <c r="B713" s="3">
-        <v>302960</v>
+        <v>327320</v>
       </c>
       <c r="C713" s="3">
         <v>0</v>
       </c>
       <c r="D713" s="3">
-        <v>9800</v>
+        <v>17640</v>
       </c>
       <c r="E713" s="3">
         <v>1960</v>
       </c>
       <c r="F713" s="3">
-        <v>314720</v>
+        <v>346920</v>
       </c>
       <c r="G713" s="3">
         <v>1960</v>
@@ -50819,25 +50819,25 @@
         <v>3454</v>
       </c>
       <c r="Q713" s="4">
-        <v>94.059</v>
+        <v>92.387</v>
       </c>
       <c r="R713" s="3">
         <v>0</v>
       </c>
       <c r="S713" s="4">
-        <v>3.043</v>
+        <v>4.979</v>
       </c>
       <c r="T713" s="4">
-        <v>0.609</v>
+        <v>0.553</v>
       </c>
       <c r="U713" s="4">
-        <v>1.217</v>
+        <v>1.106</v>
       </c>
       <c r="V713" s="3">
         <v>0</v>
       </c>
       <c r="W713" s="4">
-        <v>1.072</v>
+        <v>0.975</v>
       </c>
     </row>
   </sheetData>

</xml_diff>